<commit_message>
Worked on pin allocation
</commit_message>
<xml_diff>
--- a/hardware/SwanGanzInterface_V1.1/SwanGanzInterface_v1.1_PinAllocation.xlsx
+++ b/hardware/SwanGanzInterface_V1.1/SwanGanzInterface_v1.1_PinAllocation.xlsx
@@ -8,12 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ashto\Dev\SeniorDesign_SwanGanz\hardware\SwanGanzInterface_V1.1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{298BF75F-2E72-48DA-898C-FD02400142A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DF79EF2-ED8F-4210-97C7-C9B7E3FED79B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Pin Allocation v1.0" sheetId="1" r:id="rId1"/>
+    <sheet name="Device Comparision" sheetId="2" r:id="rId1"/>
+    <sheet name="Pin Requirements" sheetId="4" r:id="rId2"/>
+    <sheet name="PT - 48 LQFP" sheetId="5" r:id="rId3"/>
+    <sheet name="DGS28 - 28 VSSOP" sheetId="3" r:id="rId4"/>
+    <sheet name="Pin Allocation v1.0" sheetId="1" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="184">
   <si>
     <t>Pin</t>
   </si>
@@ -213,6 +217,381 @@
   </si>
   <si>
     <t>SUM :</t>
+  </si>
+  <si>
+    <t>M0G3507QPMRQ1</t>
+  </si>
+  <si>
+    <t>Part Number</t>
+  </si>
+  <si>
+    <t>M0G3507QPTRQ1</t>
+  </si>
+  <si>
+    <t>M0G3507QRGZRQ1</t>
+  </si>
+  <si>
+    <t>M0G3507QRHBRQ1</t>
+  </si>
+  <si>
+    <t>M0G3507QDGS32RQ1</t>
+  </si>
+  <si>
+    <t>M0G3507QDGS28RQ1</t>
+  </si>
+  <si>
+    <t>SRAM (KB)</t>
+  </si>
+  <si>
+    <t>Flash (KB)</t>
+  </si>
+  <si>
+    <t>ADC</t>
+  </si>
+  <si>
+    <t>ADC Channels</t>
+  </si>
+  <si>
+    <t>COMP</t>
+  </si>
+  <si>
+    <t>Number of Pins</t>
+  </si>
+  <si>
+    <t>TIMA</t>
+  </si>
+  <si>
+    <t>TIMG</t>
+  </si>
+  <si>
+    <t>GPIO</t>
+  </si>
+  <si>
+    <t>Package</t>
+  </si>
+  <si>
+    <t>64 LQFP</t>
+  </si>
+  <si>
+    <t>48 LQFP</t>
+  </si>
+  <si>
+    <t>Size</t>
+  </si>
+  <si>
+    <t>12mm x 12mm</t>
+  </si>
+  <si>
+    <t>9mm x 9mm</t>
+  </si>
+  <si>
+    <t>7mm x 7mm</t>
+  </si>
+  <si>
+    <t>5mm x 5mm</t>
+  </si>
+  <si>
+    <t>8.1mm x 4.9mm</t>
+  </si>
+  <si>
+    <t>7.1mm x 3mm</t>
+  </si>
+  <si>
+    <t>48 VQFN</t>
+  </si>
+  <si>
+    <t>32 VQFN</t>
+  </si>
+  <si>
+    <t>32 VSSOP</t>
+  </si>
+  <si>
+    <t>28 VSSOP</t>
+  </si>
+  <si>
+    <t>Pin Number</t>
+  </si>
+  <si>
+    <t>Pin Function</t>
+  </si>
+  <si>
+    <t>SGI v1.1 Funciton</t>
+  </si>
+  <si>
+    <t>PA26 / A0.1</t>
+  </si>
+  <si>
+    <t>PA27 / RTC_OUT / A0.0</t>
+  </si>
+  <si>
+    <t>VCORE</t>
+  </si>
+  <si>
+    <t>PA0</t>
+  </si>
+  <si>
+    <t>PA1</t>
+  </si>
+  <si>
+    <t>NRST</t>
+  </si>
+  <si>
+    <t>VDD</t>
+  </si>
+  <si>
+    <t>VSS</t>
+  </si>
+  <si>
+    <t>PA2 / ROSC</t>
+  </si>
+  <si>
+    <t>PA3 / LFXIN</t>
+  </si>
+  <si>
+    <t>PA4 / LFCLK_IN / LFXOUT</t>
+  </si>
+  <si>
+    <t>PA5 / HFXIN / FCC_IN</t>
+  </si>
+  <si>
+    <t>PA6 / HFCLK_IN / HFXOUT</t>
+  </si>
+  <si>
+    <t>PA9 / RTC_OUT / CLK_OUT</t>
+  </si>
+  <si>
+    <t>PA10 / CLK_OUT</t>
+  </si>
+  <si>
+    <t>PA14 / CLK_OUT / A0.12</t>
+  </si>
+  <si>
+    <t>PA15 / A1.0</t>
+  </si>
+  <si>
+    <t>PA16 / A1.1 / FCC_IN</t>
+  </si>
+  <si>
+    <t>PA17 / A1.2</t>
+  </si>
+  <si>
+    <t>PA18 / A1.3</t>
+  </si>
+  <si>
+    <t>PA19 / SWDIO</t>
+  </si>
+  <si>
+    <t>PA20 / SWCLK</t>
+  </si>
+  <si>
+    <t>PA21 / A1.7 / VREF-</t>
+  </si>
+  <si>
+    <t>PA22 / CLK_OUT / A0.7</t>
+  </si>
+  <si>
+    <t>PA23 / VREF+</t>
+  </si>
+  <si>
+    <t>PA25 / A0.2</t>
+  </si>
+  <si>
+    <t>PA24 / A0.3</t>
+  </si>
+  <si>
+    <t>Pin Name</t>
+  </si>
+  <si>
+    <t>Discription</t>
+  </si>
+  <si>
+    <t>Input for high-frequency crystal oscillator</t>
+  </si>
+  <si>
+    <t>HFXOUT</t>
+  </si>
+  <si>
+    <t>Output for high-frequency crystal oscillator</t>
+  </si>
+  <si>
+    <t>ROSC</t>
+  </si>
+  <si>
+    <t>External resistor used for improiving oscillator accuracy</t>
+  </si>
+  <si>
+    <t>QTY</t>
+  </si>
+  <si>
+    <t>Debug GPIO</t>
+  </si>
+  <si>
+    <t>Therm_ADC</t>
+  </si>
+  <si>
+    <t>P1_ADC</t>
+  </si>
+  <si>
+    <t>P2_ADC</t>
+  </si>
+  <si>
+    <t>ADC inputs for p1 circuit</t>
+  </si>
+  <si>
+    <t>ADC inputs for thermistor circuit</t>
+  </si>
+  <si>
+    <t>ADC inputs for p2 circuit</t>
+  </si>
+  <si>
+    <t>SPI SysClk for LCD driver</t>
+  </si>
+  <si>
+    <t>SPI MISO for LCD driver</t>
+  </si>
+  <si>
+    <t>LCD MOSI</t>
+  </si>
+  <si>
+    <t>SPI MOSI for LCD driver</t>
+  </si>
+  <si>
+    <t>GPIO chip select for LCD driver</t>
+  </si>
+  <si>
+    <t>GPIO reset for LCD driver</t>
+  </si>
+  <si>
+    <t>LCD_TS</t>
+  </si>
+  <si>
+    <t>ADC inputs for LCD touch screen</t>
+  </si>
+  <si>
+    <t>GPIO input specifiying the interrupt status of LCD driver</t>
+  </si>
+  <si>
+    <t>GPIO input specifiying the busy state of the LCD driver</t>
+  </si>
+  <si>
+    <t>UART_Rx</t>
+  </si>
+  <si>
+    <t>UART receive for UART to USB converter</t>
+  </si>
+  <si>
+    <t>UART_Tx</t>
+  </si>
+  <si>
+    <t>UART transmit for UART to USB converter</t>
+  </si>
+  <si>
+    <t>SW_IN</t>
+  </si>
+  <si>
+    <t>GPIO inputs for tactile switches</t>
+  </si>
+  <si>
+    <t>GPIO outputs to control LED outputs</t>
+  </si>
+  <si>
+    <t>USB_CONN</t>
+  </si>
+  <si>
+    <t>GPIO input to determine if USB is connected</t>
+  </si>
+  <si>
+    <t>GPIO outputs for debugging</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>SGI v1.1 Function</t>
+  </si>
+  <si>
+    <t>Pin Function Select</t>
+  </si>
+  <si>
+    <t>PA0 / FCC_IN</t>
+  </si>
+  <si>
+    <t>PA31 / CLK_OUT</t>
+  </si>
+  <si>
+    <t>PA3 / CMP1_OUT / LFXIN</t>
+  </si>
+  <si>
+    <t>PA7 / CLK_OUT</t>
+  </si>
+  <si>
+    <t>PB14</t>
+  </si>
+  <si>
+    <t>PA12 / FCC_IN</t>
+  </si>
+  <si>
+    <t>PB17 / A1.4</t>
+  </si>
+  <si>
+    <t>PB18 / A1.5</t>
+  </si>
+  <si>
+    <t>PB19 / A1.6</t>
+  </si>
+  <si>
+    <t>PB20 / A0.6</t>
+  </si>
+  <si>
+    <t>PB24 / A0.5</t>
+  </si>
+  <si>
+    <t>PA25 / A0.2 / OPA0_IN+</t>
+  </si>
+  <si>
+    <t>HFXTIN</t>
+  </si>
+  <si>
+    <t>TRM PAGE</t>
+  </si>
+  <si>
+    <t>TRM SECTION</t>
+  </si>
+  <si>
+    <t>2.3.1.6 High Frequency Crystal Oscillator (HFXT)</t>
+  </si>
+  <si>
+    <t>HFXIN</t>
+  </si>
+  <si>
+    <t>VREF+</t>
+  </si>
+  <si>
+    <t>VREF-</t>
+  </si>
+  <si>
+    <t>SPI0_CS0</t>
+  </si>
+  <si>
+    <t>SPI0_SCK</t>
+  </si>
+  <si>
+    <t>SPI0_POCI</t>
+  </si>
+  <si>
+    <t>SPI0_PICO</t>
+  </si>
+  <si>
+    <t>USB_Tx</t>
+  </si>
+  <si>
+    <t>USB_Rx</t>
+  </si>
+  <si>
+    <t>UART0_TX</t>
+  </si>
+  <si>
+    <t>UART0_RX</t>
   </si>
 </sst>
 </file>
@@ -228,12 +607,24 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC6C6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -248,8 +639,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -529,6 +922,1313 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7AC523F-0BD7-4B46-B60C-E63BF843905A}">
+  <dimension ref="A1:L7"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="19.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="13.7265625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.54296875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E1" t="s">
+        <v>69</v>
+      </c>
+      <c r="F1" t="s">
+        <v>70</v>
+      </c>
+      <c r="G1" t="s">
+        <v>72</v>
+      </c>
+      <c r="H1" t="s">
+        <v>73</v>
+      </c>
+      <c r="I1" t="s">
+        <v>74</v>
+      </c>
+      <c r="J1" t="s">
+        <v>71</v>
+      </c>
+      <c r="K1" t="s">
+        <v>75</v>
+      </c>
+      <c r="L1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B2">
+        <v>128</v>
+      </c>
+      <c r="C2">
+        <v>32</v>
+      </c>
+      <c r="D2">
+        <v>2</v>
+      </c>
+      <c r="E2">
+        <v>17</v>
+      </c>
+      <c r="F2">
+        <v>3</v>
+      </c>
+      <c r="G2">
+        <v>2</v>
+      </c>
+      <c r="H2">
+        <v>5</v>
+      </c>
+      <c r="I2">
+        <v>60</v>
+      </c>
+      <c r="J2">
+        <v>64</v>
+      </c>
+      <c r="K2" t="s">
+        <v>76</v>
+      </c>
+      <c r="L2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B3">
+        <v>128</v>
+      </c>
+      <c r="C3">
+        <v>32</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+      <c r="E3">
+        <v>16</v>
+      </c>
+      <c r="F3">
+        <v>3</v>
+      </c>
+      <c r="G3">
+        <v>2</v>
+      </c>
+      <c r="H3">
+        <v>5</v>
+      </c>
+      <c r="I3">
+        <v>44</v>
+      </c>
+      <c r="J3">
+        <v>48</v>
+      </c>
+      <c r="K3" t="s">
+        <v>77</v>
+      </c>
+      <c r="L3" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B4">
+        <v>128</v>
+      </c>
+      <c r="C4">
+        <v>32</v>
+      </c>
+      <c r="D4">
+        <v>2</v>
+      </c>
+      <c r="E4">
+        <v>16</v>
+      </c>
+      <c r="F4">
+        <v>3</v>
+      </c>
+      <c r="G4">
+        <v>2</v>
+      </c>
+      <c r="H4">
+        <v>5</v>
+      </c>
+      <c r="I4">
+        <v>44</v>
+      </c>
+      <c r="J4">
+        <v>48</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="L4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B5">
+        <v>128</v>
+      </c>
+      <c r="C5">
+        <v>32</v>
+      </c>
+      <c r="D5">
+        <v>2</v>
+      </c>
+      <c r="E5">
+        <v>11</v>
+      </c>
+      <c r="F5">
+        <v>3</v>
+      </c>
+      <c r="G5">
+        <v>2</v>
+      </c>
+      <c r="H5">
+        <v>5</v>
+      </c>
+      <c r="I5">
+        <v>28</v>
+      </c>
+      <c r="J5">
+        <v>32</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="L5" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>64</v>
+      </c>
+      <c r="B6">
+        <v>128</v>
+      </c>
+      <c r="C6">
+        <v>32</v>
+      </c>
+      <c r="D6">
+        <v>2</v>
+      </c>
+      <c r="E6">
+        <v>11</v>
+      </c>
+      <c r="F6">
+        <v>3</v>
+      </c>
+      <c r="G6">
+        <v>2</v>
+      </c>
+      <c r="H6">
+        <v>5</v>
+      </c>
+      <c r="I6">
+        <v>28</v>
+      </c>
+      <c r="J6">
+        <v>32</v>
+      </c>
+      <c r="K6" t="s">
+        <v>87</v>
+      </c>
+      <c r="L6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>65</v>
+      </c>
+      <c r="B7">
+        <v>128</v>
+      </c>
+      <c r="C7">
+        <v>32</v>
+      </c>
+      <c r="D7">
+        <v>2</v>
+      </c>
+      <c r="E7">
+        <v>11</v>
+      </c>
+      <c r="F7">
+        <v>3</v>
+      </c>
+      <c r="G7">
+        <v>2</v>
+      </c>
+      <c r="H7">
+        <v>5</v>
+      </c>
+      <c r="I7">
+        <v>24</v>
+      </c>
+      <c r="J7">
+        <v>28</v>
+      </c>
+      <c r="K7" t="s">
+        <v>88</v>
+      </c>
+      <c r="L7" t="s">
+        <v>84</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74AC5E4A-A5B7-4659-9F92-160B4C389A21}">
+  <dimension ref="A1:E23"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.6328125" customWidth="1"/>
+    <col min="3" max="3" width="47.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="40.6328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.54296875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>119</v>
+      </c>
+      <c r="B1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C1" t="s">
+        <v>120</v>
+      </c>
+      <c r="D1" t="s">
+        <v>171</v>
+      </c>
+      <c r="E1" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>169</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D2" t="s">
+        <v>172</v>
+      </c>
+      <c r="E2">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>122</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>123</v>
+      </c>
+      <c r="D3" t="s">
+        <v>172</v>
+      </c>
+      <c r="E3">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>124</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>128</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>129</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>130</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>49</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>136</v>
+      </c>
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="C10" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>48</v>
+      </c>
+      <c r="B11">
+        <v>1</v>
+      </c>
+      <c r="C11" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B12">
+        <v>1</v>
+      </c>
+      <c r="C12" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>55</v>
+      </c>
+      <c r="B13">
+        <v>1</v>
+      </c>
+      <c r="C13" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>47</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>140</v>
+      </c>
+      <c r="B15">
+        <v>4</v>
+      </c>
+      <c r="C15" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>144</v>
+      </c>
+      <c r="B16">
+        <v>1</v>
+      </c>
+      <c r="C16" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>146</v>
+      </c>
+      <c r="B17">
+        <v>1</v>
+      </c>
+      <c r="C17" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>151</v>
+      </c>
+      <c r="B18">
+        <v>1</v>
+      </c>
+      <c r="C18" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>148</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>40</v>
+      </c>
+      <c r="B20">
+        <v>2</v>
+      </c>
+      <c r="C20" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>127</v>
+      </c>
+      <c r="B21">
+        <v>8</v>
+      </c>
+      <c r="C21" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>154</v>
+      </c>
+      <c r="B23">
+        <f>SUM(B2:B21)</f>
+        <v>35</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6222BCFE-8BCF-40E1-9440-9F508A532375}">
+  <dimension ref="A1:D49"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.36328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B1" t="s">
+        <v>90</v>
+      </c>
+      <c r="C1" t="s">
+        <v>155</v>
+      </c>
+      <c r="D1" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>157</v>
+      </c>
+      <c r="C2" t="s">
+        <v>180</v>
+      </c>
+      <c r="D2" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>96</v>
+      </c>
+      <c r="C3" t="s">
+        <v>181</v>
+      </c>
+      <c r="D3" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>97</v>
+      </c>
+      <c r="C5" t="s">
+        <v>98</v>
+      </c>
+      <c r="D5" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>98</v>
+      </c>
+      <c r="C7" t="s">
+        <v>98</v>
+      </c>
+      <c r="D7" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>99</v>
+      </c>
+      <c r="C8" t="s">
+        <v>99</v>
+      </c>
+      <c r="D8" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>103</v>
+      </c>
+      <c r="C12" t="s">
+        <v>173</v>
+      </c>
+      <c r="D12" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>104</v>
+      </c>
+      <c r="C13" t="s">
+        <v>122</v>
+      </c>
+      <c r="D13" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>2</v>
+      </c>
+      <c r="C17" t="s">
+        <v>48</v>
+      </c>
+      <c r="D17" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>105</v>
+      </c>
+      <c r="C18" t="s">
+        <v>50</v>
+      </c>
+      <c r="D18" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>106</v>
+      </c>
+      <c r="C19" t="s">
+        <v>49</v>
+      </c>
+      <c r="D19" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>4</v>
+      </c>
+      <c r="C20" t="s">
+        <v>51</v>
+      </c>
+      <c r="D20" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A39">
+        <v>38</v>
+      </c>
+      <c r="B39" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40" t="s">
+        <v>114</v>
+      </c>
+      <c r="C40" t="s">
+        <v>175</v>
+      </c>
+      <c r="D40" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A42">
+        <v>41</v>
+      </c>
+      <c r="B42" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A43">
+        <v>42</v>
+      </c>
+      <c r="B43" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A44">
+        <v>43</v>
+      </c>
+      <c r="B44" t="s">
+        <v>116</v>
+      </c>
+      <c r="C44" t="s">
+        <v>174</v>
+      </c>
+      <c r="D44" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A45">
+        <v>44</v>
+      </c>
+      <c r="B45" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A46">
+        <v>45</v>
+      </c>
+      <c r="B46" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A47">
+        <v>46</v>
+      </c>
+      <c r="B47" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A48">
+        <v>47</v>
+      </c>
+      <c r="B48" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A49">
+        <v>48</v>
+      </c>
+      <c r="B49" t="s">
+        <v>94</v>
+      </c>
+      <c r="C49" t="s">
+        <v>94</v>
+      </c>
+      <c r="D49" t="s">
+        <v>94</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81371700-F189-4D20-B718-BFF269E87986}">
+  <dimension ref="A1:C29"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.1796875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B1" t="s">
+        <v>90</v>
+      </c>
+      <c r="C1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="s">
+        <v>117</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C37"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>

</xml_diff>

<commit_message>
Pin Allocation, updated schematic with new pins, reassigned
</commit_message>
<xml_diff>
--- a/hardware/SwanGanzInterface_V1.1/SwanGanzInterface_v1.1_PinAllocation.xlsx
+++ b/hardware/SwanGanzInterface_V1.1/SwanGanzInterface_v1.1_PinAllocation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ashto\Dev\SeniorDesign_SwanGanz\hardware\SwanGanzInterface_V1.1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A867E3C-7FBA-4387-872A-357911B968F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{220E54C6-0FA3-4802-821C-84AF49EFE1E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Device Comparision" sheetId="2" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="224">
   <si>
     <t>Pin</t>
   </si>
@@ -570,33 +570,12 @@
     <t>VREF-</t>
   </si>
   <si>
-    <t>SPI0_CS0</t>
-  </si>
-  <si>
-    <t>SPI0_SCK</t>
-  </si>
-  <si>
-    <t>SPI0_POCI</t>
-  </si>
-  <si>
-    <t>SPI0_PICO</t>
-  </si>
-  <si>
     <t>USB_Tx</t>
   </si>
   <si>
     <t>USB_Rx</t>
   </si>
   <si>
-    <t>UART0_TX</t>
-  </si>
-  <si>
-    <t>UART0_RX</t>
-  </si>
-  <si>
-    <t>LCD_RESET</t>
-  </si>
-  <si>
     <t>GPIO - Input</t>
   </si>
   <si>
@@ -642,12 +621,6 @@
     <t>PT - Assigned</t>
   </si>
   <si>
-    <t>y</t>
-  </si>
-  <si>
-    <t>A1.0</t>
-  </si>
-  <si>
     <t>A1.2</t>
   </si>
   <si>
@@ -669,30 +642,6 @@
     <t>A1.1</t>
   </si>
   <si>
-    <t>DEBUG1</t>
-  </si>
-  <si>
-    <t>DEBUG2</t>
-  </si>
-  <si>
-    <t>DEBUG3</t>
-  </si>
-  <si>
-    <t>DEBUG4</t>
-  </si>
-  <si>
-    <t>DEBUG5</t>
-  </si>
-  <si>
-    <t>DEBUG6</t>
-  </si>
-  <si>
-    <t>DEBUG7</t>
-  </si>
-  <si>
-    <t>DEBUG8</t>
-  </si>
-  <si>
     <t>LED_WORKING</t>
   </si>
   <si>
@@ -703,6 +652,66 @@
   </si>
   <si>
     <t>Serial wire debug data input/output</t>
+  </si>
+  <si>
+    <t>SPI1_SCK</t>
+  </si>
+  <si>
+    <t>SPI1_PICO</t>
+  </si>
+  <si>
+    <t>LCD_PICO</t>
+  </si>
+  <si>
+    <t>SPI1_POIC</t>
+  </si>
+  <si>
+    <t>LCD_POCI</t>
+  </si>
+  <si>
+    <t>SPI1_CS0</t>
+  </si>
+  <si>
+    <t>UART1_TX</t>
+  </si>
+  <si>
+    <t>UART1_RX</t>
+  </si>
+  <si>
+    <t>DEBUG 1</t>
+  </si>
+  <si>
+    <t>DEBUG 2</t>
+  </si>
+  <si>
+    <t>DEBUG 3</t>
+  </si>
+  <si>
+    <t>DEBUG 4</t>
+  </si>
+  <si>
+    <t>DEBUG 5</t>
+  </si>
+  <si>
+    <t>DEBUG 6</t>
+  </si>
+  <si>
+    <t>DEBUG 7</t>
+  </si>
+  <si>
+    <t>DEBUG 8</t>
+  </si>
+  <si>
+    <t>GPIO OUTPUT</t>
+  </si>
+  <si>
+    <t>DAC</t>
+  </si>
+  <si>
+    <t>SPEAKER</t>
+  </si>
+  <si>
+    <t>A1.6</t>
   </si>
 </sst>
 </file>
@@ -1349,7 +1358,7 @@
         <v>170</v>
       </c>
       <c r="F1" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
@@ -1368,9 +1377,7 @@
       <c r="E2">
         <v>231</v>
       </c>
-      <c r="F2" s="3" t="s">
-        <v>200</v>
-      </c>
+      <c r="F2" s="3"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
@@ -1388,9 +1395,7 @@
       <c r="E3">
         <v>231</v>
       </c>
-      <c r="F3" s="3" t="s">
-        <v>200</v>
-      </c>
+      <c r="F3" s="3"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
@@ -1402,9 +1407,7 @@
       <c r="C4" t="s">
         <v>125</v>
       </c>
-      <c r="F4" s="3" t="s">
-        <v>200</v>
-      </c>
+      <c r="F4" s="3"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
@@ -1416,9 +1419,7 @@
       <c r="C5" t="s">
         <v>132</v>
       </c>
-      <c r="F5" s="3" t="s">
-        <v>200</v>
-      </c>
+      <c r="F5" s="3"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
@@ -1430,9 +1431,7 @@
       <c r="C6" t="s">
         <v>131</v>
       </c>
-      <c r="F6" s="3" t="s">
-        <v>200</v>
-      </c>
+      <c r="F6" s="3"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
@@ -1444,9 +1443,7 @@
       <c r="C7" t="s">
         <v>133</v>
       </c>
-      <c r="F7" s="3" t="s">
-        <v>200</v>
-      </c>
+      <c r="F7" s="3"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
@@ -1458,9 +1455,7 @@
       <c r="C8" t="s">
         <v>134</v>
       </c>
-      <c r="F8" s="3" t="s">
-        <v>200</v>
-      </c>
+      <c r="F8" s="3"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
@@ -1472,9 +1467,7 @@
       <c r="C9" t="s">
         <v>135</v>
       </c>
-      <c r="F9" s="3" t="s">
-        <v>200</v>
-      </c>
+      <c r="F9" s="3"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
@@ -1486,9 +1479,7 @@
       <c r="C10" t="s">
         <v>137</v>
       </c>
-      <c r="F10" s="3" t="s">
-        <v>200</v>
-      </c>
+      <c r="F10" s="3"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
@@ -1500,9 +1491,7 @@
       <c r="C11" t="s">
         <v>138</v>
       </c>
-      <c r="F11" s="3" t="s">
-        <v>200</v>
-      </c>
+      <c r="F11" s="3"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
@@ -1514,9 +1503,7 @@
       <c r="C12" t="s">
         <v>139</v>
       </c>
-      <c r="F12" s="3" t="s">
-        <v>200</v>
-      </c>
+      <c r="F12" s="3"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
@@ -1528,9 +1515,7 @@
       <c r="C13" t="s">
         <v>143</v>
       </c>
-      <c r="F13" s="3" t="s">
-        <v>200</v>
-      </c>
+      <c r="F13" s="3"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
@@ -1542,9 +1527,7 @@
       <c r="C14" t="s">
         <v>142</v>
       </c>
-      <c r="F14" s="3" t="s">
-        <v>200</v>
-      </c>
+      <c r="F14" s="3"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
@@ -1556,9 +1539,7 @@
       <c r="C15" t="s">
         <v>141</v>
       </c>
-      <c r="F15" s="3" t="s">
-        <v>200</v>
-      </c>
+      <c r="F15" s="3"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
@@ -1570,9 +1551,7 @@
       <c r="C16" t="s">
         <v>145</v>
       </c>
-      <c r="F16" s="3" t="s">
-        <v>200</v>
-      </c>
+      <c r="F16" s="3"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
@@ -1584,9 +1563,7 @@
       <c r="C17" t="s">
         <v>147</v>
       </c>
-      <c r="F17" s="3" t="s">
-        <v>200</v>
-      </c>
+      <c r="F17" s="3"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
@@ -1598,9 +1575,7 @@
       <c r="C18" t="s">
         <v>152</v>
       </c>
-      <c r="F18" s="3" t="s">
-        <v>200</v>
-      </c>
+      <c r="F18" s="3"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
@@ -1624,9 +1599,7 @@
       <c r="C20" t="s">
         <v>150</v>
       </c>
-      <c r="F20" s="3" t="s">
-        <v>200</v>
-      </c>
+      <c r="F20" s="3"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
@@ -1638,37 +1611,31 @@
       <c r="C21" t="s">
         <v>153</v>
       </c>
-      <c r="F21" s="3" t="s">
-        <v>200</v>
-      </c>
+      <c r="F21" s="3"/>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>205</v>
+        <v>196</v>
       </c>
       <c r="B22">
         <v>1</v>
       </c>
       <c r="C22" t="s">
-        <v>219</v>
-      </c>
-      <c r="F22" s="3" t="s">
-        <v>200</v>
-      </c>
+        <v>202</v>
+      </c>
+      <c r="F22" s="3"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>204</v>
+        <v>195</v>
       </c>
       <c r="B23">
         <v>1</v>
       </c>
       <c r="C23" t="s">
-        <v>220</v>
-      </c>
-      <c r="F23" s="3" t="s">
-        <v>200</v>
-      </c>
+        <v>203</v>
+      </c>
+      <c r="F23" s="3"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
@@ -1716,12 +1683,6 @@
       <c r="B2" t="s">
         <v>157</v>
       </c>
-      <c r="C2" t="s">
-        <v>180</v>
-      </c>
-      <c r="D2" t="s">
-        <v>182</v>
-      </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3">
@@ -1730,12 +1691,6 @@
       <c r="B3" t="s">
         <v>96</v>
       </c>
-      <c r="C3" t="s">
-        <v>181</v>
-      </c>
-      <c r="D3" t="s">
-        <v>183</v>
-      </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4">
@@ -1744,12 +1699,6 @@
       <c r="B4" t="s">
         <v>16</v>
       </c>
-      <c r="C4" t="s">
-        <v>151</v>
-      </c>
-      <c r="D4" t="s">
-        <v>185</v>
-      </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5">
@@ -1822,6 +1771,12 @@
       <c r="B10" t="s">
         <v>159</v>
       </c>
+      <c r="C10" t="s">
+        <v>52</v>
+      </c>
+      <c r="D10" t="s">
+        <v>178</v>
+      </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11">
@@ -1830,6 +1785,12 @@
       <c r="B11" t="s">
         <v>102</v>
       </c>
+      <c r="C11" t="s">
+        <v>53</v>
+      </c>
+      <c r="D11" t="s">
+        <v>178</v>
+      </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12">
@@ -1867,10 +1828,10 @@
         <v>160</v>
       </c>
       <c r="C14" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="D14" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
@@ -1881,10 +1842,10 @@
         <v>20</v>
       </c>
       <c r="C15" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="D15" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
@@ -1895,10 +1856,10 @@
         <v>22</v>
       </c>
       <c r="C16" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="D16" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
@@ -1909,10 +1870,10 @@
         <v>2</v>
       </c>
       <c r="C17" t="s">
-        <v>48</v>
+        <v>176</v>
       </c>
       <c r="D17" t="s">
-        <v>176</v>
+        <v>210</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
@@ -1923,10 +1884,10 @@
         <v>105</v>
       </c>
       <c r="C18" t="s">
-        <v>50</v>
+        <v>177</v>
       </c>
       <c r="D18" t="s">
-        <v>179</v>
+        <v>211</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
@@ -1937,7 +1898,7 @@
         <v>106</v>
       </c>
       <c r="C19" t="s">
-        <v>49</v>
+        <v>151</v>
       </c>
       <c r="D19" t="s">
         <v>178</v>
@@ -1951,10 +1912,10 @@
         <v>4</v>
       </c>
       <c r="C20" t="s">
-        <v>51</v>
+        <v>215</v>
       </c>
       <c r="D20" t="s">
-        <v>177</v>
+        <v>220</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
@@ -1965,10 +1926,10 @@
         <v>24</v>
       </c>
       <c r="C21" t="s">
-        <v>184</v>
+        <v>48</v>
       </c>
       <c r="D21" t="s">
-        <v>186</v>
+        <v>209</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
@@ -1979,10 +1940,10 @@
         <v>25</v>
       </c>
       <c r="C22" t="s">
-        <v>55</v>
+        <v>208</v>
       </c>
       <c r="D22" t="s">
-        <v>185</v>
+        <v>207</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
@@ -1993,10 +1954,10 @@
         <v>26</v>
       </c>
       <c r="C23" t="s">
-        <v>47</v>
+        <v>206</v>
       </c>
       <c r="D23" t="s">
-        <v>185</v>
+        <v>205</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.35">
@@ -2007,10 +1968,10 @@
         <v>27</v>
       </c>
       <c r="C24" t="s">
-        <v>212</v>
+        <v>51</v>
       </c>
       <c r="D24" t="s">
-        <v>186</v>
+        <v>204</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
@@ -2021,10 +1982,10 @@
         <v>161</v>
       </c>
       <c r="C25" t="s">
-        <v>213</v>
+        <v>55</v>
       </c>
       <c r="D25" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.35">
@@ -2035,10 +1996,10 @@
         <v>30</v>
       </c>
       <c r="C26" t="s">
-        <v>214</v>
+        <v>54</v>
       </c>
       <c r="D26" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.35">
@@ -2049,10 +2010,10 @@
         <v>31</v>
       </c>
       <c r="C27" t="s">
-        <v>215</v>
+        <v>47</v>
       </c>
       <c r="D27" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.35">
@@ -2066,7 +2027,7 @@
         <v>216</v>
       </c>
       <c r="D28" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.35">
@@ -2076,6 +2037,12 @@
       <c r="B29" t="s">
         <v>6</v>
       </c>
+      <c r="C29" t="s">
+        <v>217</v>
+      </c>
+      <c r="D29" t="s">
+        <v>179</v>
+      </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30">
@@ -2084,6 +2051,12 @@
       <c r="B30" t="s">
         <v>107</v>
       </c>
+      <c r="C30" t="s">
+        <v>218</v>
+      </c>
+      <c r="D30" t="s">
+        <v>179</v>
+      </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31">
@@ -2093,10 +2066,10 @@
         <v>108</v>
       </c>
       <c r="C31" t="s">
-        <v>46</v>
+        <v>222</v>
       </c>
       <c r="D31" t="s">
-        <v>201</v>
+        <v>221</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.35">
@@ -2107,10 +2080,10 @@
         <v>109</v>
       </c>
       <c r="C32" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="D32" t="s">
-        <v>208</v>
+        <v>199</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.35">
@@ -2121,10 +2094,10 @@
         <v>110</v>
       </c>
       <c r="C33" t="s">
-        <v>195</v>
+        <v>43</v>
       </c>
       <c r="D33" t="s">
-        <v>202</v>
+        <v>193</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.35">
@@ -2135,10 +2108,10 @@
         <v>111</v>
       </c>
       <c r="C34" t="s">
-        <v>197</v>
+        <v>188</v>
       </c>
       <c r="D34" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.35">
@@ -2149,10 +2122,10 @@
         <v>112</v>
       </c>
       <c r="C35" t="s">
-        <v>204</v>
+        <v>195</v>
       </c>
       <c r="D35" t="s">
-        <v>204</v>
+        <v>195</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.35">
@@ -2163,10 +2136,10 @@
         <v>113</v>
       </c>
       <c r="C36" t="s">
-        <v>205</v>
+        <v>196</v>
       </c>
       <c r="D36" t="s">
-        <v>205</v>
+        <v>196</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.35">
@@ -2177,10 +2150,10 @@
         <v>163</v>
       </c>
       <c r="C37" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="D37" t="s">
-        <v>206</v>
+        <v>197</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.35">
@@ -2191,10 +2164,10 @@
         <v>164</v>
       </c>
       <c r="C38" t="s">
+        <v>189</v>
+      </c>
+      <c r="D38" t="s">
         <v>198</v>
-      </c>
-      <c r="D38" t="s">
-        <v>207</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.35">
@@ -2204,6 +2177,12 @@
       <c r="B39" t="s">
         <v>165</v>
       </c>
+      <c r="C39" t="s">
+        <v>191</v>
+      </c>
+      <c r="D39" t="s">
+        <v>223</v>
+      </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A40">
@@ -2227,10 +2206,10 @@
         <v>115</v>
       </c>
       <c r="C41" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D41" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.35">
@@ -2241,10 +2220,10 @@
         <v>166</v>
       </c>
       <c r="C42" t="s">
-        <v>218</v>
+        <v>200</v>
       </c>
       <c r="D42" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.35">
@@ -2254,6 +2233,12 @@
       <c r="B43" t="s">
         <v>167</v>
       </c>
+      <c r="C43" t="s">
+        <v>201</v>
+      </c>
+      <c r="D43" t="s">
+        <v>179</v>
+      </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A44">
@@ -2277,10 +2262,10 @@
         <v>118</v>
       </c>
       <c r="C45" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="D45" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.35">
@@ -2291,10 +2276,10 @@
         <v>168</v>
       </c>
       <c r="C46" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="D46" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.35">
@@ -2305,10 +2290,10 @@
         <v>92</v>
       </c>
       <c r="C47" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="D47" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.35">
@@ -2319,10 +2304,10 @@
         <v>93</v>
       </c>
       <c r="C48" t="s">
+        <v>180</v>
+      </c>
+      <c r="D48" t="s">
         <v>187</v>
-      </c>
-      <c r="D48" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Worked on FT232R circuit - RTS, CTS etc
</commit_message>
<xml_diff>
--- a/hardware/SwanGanzInterface_V1.1/SwanGanzInterface_v1.1_PinAllocation.xlsx
+++ b/hardware/SwanGanzInterface_V1.1/SwanGanzInterface_v1.1_PinAllocation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ashto\Dev\SeniorDesign_SwanGanz\hardware\SwanGanzInterface_V1.1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{220E54C6-0FA3-4802-821C-84AF49EFE1E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{361EA152-DB38-4BF7-A4F5-C8A01A7E9E4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="228">
   <si>
     <t>Pin</t>
   </si>
@@ -678,15 +678,6 @@
     <t>UART1_RX</t>
   </si>
   <si>
-    <t>DEBUG 1</t>
-  </si>
-  <si>
-    <t>DEBUG 2</t>
-  </si>
-  <si>
-    <t>DEBUG 3</t>
-  </si>
-  <si>
     <t>DEBUG 4</t>
   </si>
   <si>
@@ -712,6 +703,27 @@
   </si>
   <si>
     <t>A1.6</t>
+  </si>
+  <si>
+    <t>USB_CTS</t>
+  </si>
+  <si>
+    <t>UART1_CTS</t>
+  </si>
+  <si>
+    <t>UART1_RTS</t>
+  </si>
+  <si>
+    <t>USB_RTS</t>
+  </si>
+  <si>
+    <t>DEBUG1</t>
+  </si>
+  <si>
+    <t>DEBUG2</t>
+  </si>
+  <si>
+    <t>DEBUG3</t>
   </si>
 </sst>
 </file>
@@ -1699,6 +1711,12 @@
       <c r="B4" t="s">
         <v>16</v>
       </c>
+      <c r="C4" t="s">
+        <v>225</v>
+      </c>
+      <c r="D4" t="s">
+        <v>179</v>
+      </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5">
@@ -1721,6 +1739,12 @@
       <c r="B6" t="s">
         <v>158</v>
       </c>
+      <c r="C6" t="s">
+        <v>226</v>
+      </c>
+      <c r="D6" t="s">
+        <v>179</v>
+      </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7">
@@ -1828,7 +1852,7 @@
         <v>160</v>
       </c>
       <c r="C14" t="s">
-        <v>212</v>
+        <v>227</v>
       </c>
       <c r="D14" t="s">
         <v>179</v>
@@ -1842,10 +1866,10 @@
         <v>20</v>
       </c>
       <c r="C15" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="D15" t="s">
-        <v>179</v>
+        <v>222</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
@@ -1856,10 +1880,10 @@
         <v>22</v>
       </c>
       <c r="C16" t="s">
-        <v>214</v>
+        <v>224</v>
       </c>
       <c r="D16" t="s">
-        <v>179</v>
+        <v>223</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
@@ -1912,10 +1936,10 @@
         <v>4</v>
       </c>
       <c r="C20" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="D20" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
@@ -2024,7 +2048,7 @@
         <v>162</v>
       </c>
       <c r="C28" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="D28" t="s">
         <v>179</v>
@@ -2038,7 +2062,7 @@
         <v>6</v>
       </c>
       <c r="C29" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="D29" t="s">
         <v>179</v>
@@ -2052,7 +2076,7 @@
         <v>107</v>
       </c>
       <c r="C30" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="D30" t="s">
         <v>179</v>
@@ -2066,10 +2090,10 @@
         <v>108</v>
       </c>
       <c r="C31" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="D31" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.35">
@@ -2181,7 +2205,7 @@
         <v>191</v>
       </c>
       <c r="D39" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.35">
@@ -2206,7 +2230,7 @@
         <v>115</v>
       </c>
       <c r="C41" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="D41" t="s">
         <v>179</v>

</xml_diff>

<commit_message>
Started converting things to use touch screen chip
</commit_message>
<xml_diff>
--- a/hardware/SwanGanzInterface_V1.1/SwanGanzInterface_v1.1_PinAllocation.xlsx
+++ b/hardware/SwanGanzInterface_V1.1/SwanGanzInterface_v1.1_PinAllocation.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ashto\Dev\SeniorDesign_SwanGanz\hardware\SwanGanzInterface_V1.1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{361EA152-DB38-4BF7-A4F5-C8A01A7E9E4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FCB407C-047D-4B8F-8BB5-EF9BD8170BF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="229">
   <si>
     <t>Pin</t>
   </si>
@@ -582,24 +582,6 @@
     <t>GPIO - Output</t>
   </si>
   <si>
-    <t>LCD_Y-</t>
-  </si>
-  <si>
-    <t>LCD_Y+</t>
-  </si>
-  <si>
-    <t>LCD_X+</t>
-  </si>
-  <si>
-    <t>LCD_X-</t>
-  </si>
-  <si>
-    <t>A0.2</t>
-  </si>
-  <si>
-    <t>A0.3</t>
-  </si>
-  <si>
     <t>A0.1</t>
   </si>
   <si>
@@ -621,9 +603,6 @@
     <t>PT - Assigned</t>
   </si>
   <si>
-    <t>A1.2</t>
-  </si>
-  <si>
     <t>A1.3</t>
   </si>
   <si>
@@ -639,9 +618,6 @@
     <t>A1.5</t>
   </si>
   <si>
-    <t>A1.1</t>
-  </si>
-  <si>
     <t>LED_WORKING</t>
   </si>
   <si>
@@ -724,6 +700,33 @@
   </si>
   <si>
     <t>DEBUG3</t>
+  </si>
+  <si>
+    <t>TOUCH_SCK</t>
+  </si>
+  <si>
+    <t>TOUCH_PICO</t>
+  </si>
+  <si>
+    <t>SPI0_SCK</t>
+  </si>
+  <si>
+    <t>SPI0_POCI</t>
+  </si>
+  <si>
+    <t>TOUCH_POCI</t>
+  </si>
+  <si>
+    <t>SPI0_PICO</t>
+  </si>
+  <si>
+    <t>TOUCH_CS</t>
+  </si>
+  <si>
+    <t>SPI0_CS3</t>
+  </si>
+  <si>
+    <t>PENIRQ</t>
   </si>
 </sst>
 </file>
@@ -1370,7 +1373,7 @@
         <v>170</v>
       </c>
       <c r="F1" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
@@ -1627,25 +1630,25 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="B22">
         <v>1</v>
       </c>
       <c r="C22" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="F22" s="3"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
+        <v>188</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
         <v>195</v>
-      </c>
-      <c r="B23">
-        <v>1</v>
-      </c>
-      <c r="C23" t="s">
-        <v>203</v>
       </c>
       <c r="F23" s="3"/>
     </row>
@@ -1665,7 +1668,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6222BCFE-8BCF-40E1-9440-9F508A532375}">
-  <dimension ref="A1:D49"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.6328125" bestFit="1" customWidth="1"/>
@@ -1712,7 +1715,7 @@
         <v>16</v>
       </c>
       <c r="C4" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
       <c r="D4" t="s">
         <v>179</v>
@@ -1740,7 +1743,7 @@
         <v>158</v>
       </c>
       <c r="C6" t="s">
-        <v>226</v>
+        <v>218</v>
       </c>
       <c r="D6" t="s">
         <v>179</v>
@@ -1852,7 +1855,7 @@
         <v>160</v>
       </c>
       <c r="C14" t="s">
-        <v>227</v>
+        <v>219</v>
       </c>
       <c r="D14" t="s">
         <v>179</v>
@@ -1866,10 +1869,10 @@
         <v>20</v>
       </c>
       <c r="C15" t="s">
-        <v>221</v>
+        <v>213</v>
       </c>
       <c r="D15" t="s">
-        <v>222</v>
+        <v>214</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
@@ -1880,13 +1883,13 @@
         <v>22</v>
       </c>
       <c r="C16" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="D16" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1897,10 +1900,10 @@
         <v>176</v>
       </c>
       <c r="D17" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1911,10 +1914,10 @@
         <v>177</v>
       </c>
       <c r="D18" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1928,7 +1931,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1936,13 +1939,13 @@
         <v>4</v>
       </c>
       <c r="C20" t="s">
-        <v>212</v>
+        <v>204</v>
       </c>
       <c r="D20" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1953,10 +1956,10 @@
         <v>48</v>
       </c>
       <c r="D21" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1964,13 +1967,13 @@
         <v>25</v>
       </c>
       <c r="C22" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="D22" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1978,13 +1981,13 @@
         <v>26</v>
       </c>
       <c r="C23" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="D23" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1995,10 +1998,10 @@
         <v>51</v>
       </c>
       <c r="D24" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>24</v>
       </c>
@@ -2012,7 +2015,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>25</v>
       </c>
@@ -2026,7 +2029,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>26</v>
       </c>
@@ -2040,7 +2043,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>27</v>
       </c>
@@ -2048,13 +2051,19 @@
         <v>162</v>
       </c>
       <c r="C28" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
       <c r="D28" t="s">
+        <v>222</v>
+      </c>
+      <c r="F28" t="s">
+        <v>205</v>
+      </c>
+      <c r="G28" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>28</v>
       </c>
@@ -2062,13 +2071,19 @@
         <v>6</v>
       </c>
       <c r="C29" t="s">
-        <v>214</v>
+        <v>224</v>
       </c>
       <c r="D29" t="s">
+        <v>223</v>
+      </c>
+      <c r="F29" t="s">
+        <v>206</v>
+      </c>
+      <c r="G29" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>29</v>
       </c>
@@ -2076,13 +2091,19 @@
         <v>107</v>
       </c>
       <c r="C30" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="D30" t="s">
+        <v>225</v>
+      </c>
+      <c r="F30" t="s">
+        <v>207</v>
+      </c>
+      <c r="G30" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>30</v>
       </c>
@@ -2090,13 +2111,13 @@
         <v>108</v>
       </c>
       <c r="C31" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="D31" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>31</v>
       </c>
@@ -2104,10 +2125,10 @@
         <v>109</v>
       </c>
       <c r="C32" t="s">
-        <v>46</v>
+        <v>228</v>
       </c>
       <c r="D32" t="s">
-        <v>199</v>
+        <v>178</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.35">
@@ -2117,12 +2138,6 @@
       <c r="B33" t="s">
         <v>110</v>
       </c>
-      <c r="C33" t="s">
-        <v>43</v>
-      </c>
-      <c r="D33" t="s">
-        <v>193</v>
-      </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34">
@@ -2132,10 +2147,10 @@
         <v>111</v>
       </c>
       <c r="C34" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="D34" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.35">
@@ -2146,10 +2161,10 @@
         <v>112</v>
       </c>
       <c r="C35" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="D35" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.35">
@@ -2160,10 +2175,10 @@
         <v>113</v>
       </c>
       <c r="C36" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="D36" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.35">
@@ -2174,10 +2189,10 @@
         <v>163</v>
       </c>
       <c r="C37" t="s">
+        <v>184</v>
+      </c>
+      <c r="D37" t="s">
         <v>190</v>
-      </c>
-      <c r="D37" t="s">
-        <v>197</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.35">
@@ -2188,10 +2203,10 @@
         <v>164</v>
       </c>
       <c r="C38" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="D38" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.35">
@@ -2202,10 +2217,10 @@
         <v>165</v>
       </c>
       <c r="C39" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="D39" t="s">
-        <v>220</v>
+        <v>212</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.35">
@@ -2230,7 +2245,7 @@
         <v>115</v>
       </c>
       <c r="C41" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="D41" t="s">
         <v>179</v>
@@ -2244,7 +2259,7 @@
         <v>166</v>
       </c>
       <c r="C42" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="D42" t="s">
         <v>179</v>
@@ -2258,7 +2273,7 @@
         <v>167</v>
       </c>
       <c r="C43" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="D43" t="s">
         <v>179</v>
@@ -2286,10 +2301,10 @@
         <v>118</v>
       </c>
       <c r="C45" t="s">
-        <v>182</v>
+        <v>226</v>
       </c>
       <c r="D45" t="s">
-        <v>185</v>
+        <v>227</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.35">
@@ -2299,12 +2314,6 @@
       <c r="B46" t="s">
         <v>168</v>
       </c>
-      <c r="C46" t="s">
-        <v>183</v>
-      </c>
-      <c r="D46" t="s">
-        <v>184</v>
-      </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A47">
@@ -2314,10 +2323,10 @@
         <v>92</v>
       </c>
       <c r="C47" t="s">
-        <v>181</v>
+        <v>43</v>
       </c>
       <c r="D47" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.35">
@@ -2328,10 +2337,10 @@
         <v>93</v>
       </c>
       <c r="C48" t="s">
-        <v>180</v>
+        <v>46</v>
       </c>
       <c r="D48" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Added lots, moving to 64 pin micro
</commit_message>
<xml_diff>
--- a/hardware/SwanGanzInterface_V1.1/SwanGanzInterface_v1.1_PinAllocation.xlsx
+++ b/hardware/SwanGanzInterface_V1.1/SwanGanzInterface_v1.1_PinAllocation.xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ashto\Dev\SeniorDesign_SwanGanz\hardware\SwanGanzInterface_V1.1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FCB407C-047D-4B8F-8BB5-EF9BD8170BF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3F70114-8A99-475F-A5AB-4C7D0031B5BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="12980" windowHeight="15370" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Device Comparision" sheetId="2" r:id="rId1"/>
     <sheet name="Pin Requirements" sheetId="4" r:id="rId2"/>
-    <sheet name="PT - 48 LQFP" sheetId="5" r:id="rId3"/>
-    <sheet name="DGS28 - 28 VSSOP" sheetId="3" r:id="rId4"/>
-    <sheet name="Pin Allocation v1.0" sheetId="1" r:id="rId5"/>
+    <sheet name="PM - 64 LQFP" sheetId="6" r:id="rId3"/>
+    <sheet name="PT - 48 LQFP" sheetId="5" r:id="rId4"/>
+    <sheet name="DGS28 - 28 VSSOP" sheetId="3" r:id="rId5"/>
+    <sheet name="Pin Allocation v1.0" sheetId="1" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="246">
   <si>
     <t>Pin</t>
   </si>
@@ -727,6 +728,57 @@
   </si>
   <si>
     <t>PENIRQ</t>
+  </si>
+  <si>
+    <t>PB18 / 1.5</t>
+  </si>
+  <si>
+    <t>PB21</t>
+  </si>
+  <si>
+    <t>PB22</t>
+  </si>
+  <si>
+    <t>PA23 / A0.3</t>
+  </si>
+  <si>
+    <t>PB25 / A0.4</t>
+  </si>
+  <si>
+    <t>PB26</t>
+  </si>
+  <si>
+    <t>PB27</t>
+  </si>
+  <si>
+    <t>PA27 / A0.0</t>
+  </si>
+  <si>
+    <t>PA29</t>
+  </si>
+  <si>
+    <t>PA30</t>
+  </si>
+  <si>
+    <t>PB5</t>
+  </si>
+  <si>
+    <t>PB10</t>
+  </si>
+  <si>
+    <t>PB11 / CLK_OUT</t>
+  </si>
+  <si>
+    <t>SPI1_POCI</t>
+  </si>
+  <si>
+    <t>SPI11_SCK</t>
+  </si>
+  <si>
+    <t>SPI0_CS0</t>
+  </si>
+  <si>
+    <t>Translated</t>
   </si>
 </sst>
 </file>
@@ -742,7 +794,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -761,6 +813,24 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -774,13 +844,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1667,6 +1740,613 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D113DCF4-3EF2-4E93-9D02-C93F34579EEA}">
+  <dimension ref="A1:D65"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="23.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.36328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>90</v>
+      </c>
+      <c r="C1" t="s">
+        <v>155</v>
+      </c>
+      <c r="D1" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="2">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="2">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="2">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="2">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="2">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="2">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" s="2">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" s="2">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" s="2">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" s="2">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" s="2">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" s="2">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" s="2">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A17" s="2">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A18" s="4">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A19" s="4">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A20" s="4">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A21" s="4">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A22" s="4">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A23" s="4">
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A24" s="4">
+        <v>23</v>
+      </c>
+      <c r="B24" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A25" s="4">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A26" s="4">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A27" s="4">
+        <v>26</v>
+      </c>
+      <c r="B27" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A28" s="4">
+        <v>27</v>
+      </c>
+      <c r="B28" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A29" s="4">
+        <v>28</v>
+      </c>
+      <c r="B29" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A30" s="4">
+        <v>29</v>
+      </c>
+      <c r="B30" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A31" s="4">
+        <v>30</v>
+      </c>
+      <c r="B31" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A32" s="4">
+        <v>31</v>
+      </c>
+      <c r="B32" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A33" s="4">
+        <v>32</v>
+      </c>
+      <c r="B33" t="s">
+        <v>94</v>
+      </c>
+      <c r="C33" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A34" s="6">
+        <v>33</v>
+      </c>
+      <c r="B34" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A35" s="6">
+        <v>34</v>
+      </c>
+      <c r="B35" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A36" s="6">
+        <v>35</v>
+      </c>
+      <c r="B36" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A37" s="6">
+        <v>36</v>
+      </c>
+      <c r="B37" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A38" s="6">
+        <v>37</v>
+      </c>
+      <c r="B38" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A39" s="6">
+        <v>38</v>
+      </c>
+      <c r="B39" t="s">
+        <v>97</v>
+      </c>
+      <c r="C39" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A40" s="6">
+        <v>39</v>
+      </c>
+      <c r="B40" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A41" s="6">
+        <v>40</v>
+      </c>
+      <c r="B41" t="s">
+        <v>98</v>
+      </c>
+      <c r="C41" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A42" s="6">
+        <v>41</v>
+      </c>
+      <c r="B42" t="s">
+        <v>99</v>
+      </c>
+      <c r="C42" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A43" s="6">
+        <v>42</v>
+      </c>
+      <c r="B43" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A44" s="6">
+        <v>43</v>
+      </c>
+      <c r="B44" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A45" s="6">
+        <v>44</v>
+      </c>
+      <c r="B45" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A46" s="6">
+        <v>45</v>
+      </c>
+      <c r="B46" t="s">
+        <v>103</v>
+      </c>
+      <c r="C46" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A47" s="6">
+        <v>46</v>
+      </c>
+      <c r="B47" t="s">
+        <v>104</v>
+      </c>
+      <c r="C47" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A48" s="6">
+        <v>47</v>
+      </c>
+      <c r="B48" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A49" s="6">
+        <v>48</v>
+      </c>
+      <c r="B49" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A50" s="5">
+        <v>49</v>
+      </c>
+      <c r="B50" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A51" s="5">
+        <v>50</v>
+      </c>
+      <c r="B51" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A52" s="5">
+        <v>51</v>
+      </c>
+      <c r="B52" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A53" s="5">
+        <v>52</v>
+      </c>
+      <c r="B53" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A54" s="5">
+        <v>53</v>
+      </c>
+      <c r="B54" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A55" s="5">
+        <v>54</v>
+      </c>
+      <c r="B55" t="s">
+        <v>2</v>
+      </c>
+      <c r="C55" t="s">
+        <v>226</v>
+      </c>
+      <c r="D55" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A56" s="5">
+        <v>55</v>
+      </c>
+      <c r="B56" t="s">
+        <v>105</v>
+      </c>
+      <c r="C56" t="s">
+        <v>221</v>
+      </c>
+      <c r="D56" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A57" s="5">
+        <v>56</v>
+      </c>
+      <c r="B57" t="s">
+        <v>106</v>
+      </c>
+      <c r="C57" t="s">
+        <v>224</v>
+      </c>
+      <c r="D57" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A58" s="5">
+        <v>57</v>
+      </c>
+      <c r="B58" t="s">
+        <v>4</v>
+      </c>
+      <c r="C58" t="s">
+        <v>220</v>
+      </c>
+      <c r="D58" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A59" s="5">
+        <v>58</v>
+      </c>
+      <c r="B59" t="s">
+        <v>24</v>
+      </c>
+      <c r="C59" t="s">
+        <v>48</v>
+      </c>
+      <c r="D59" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A60" s="5">
+        <v>59</v>
+      </c>
+      <c r="B60" t="s">
+        <v>25</v>
+      </c>
+      <c r="C60" t="s">
+        <v>200</v>
+      </c>
+      <c r="D60" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A61" s="5">
+        <v>60</v>
+      </c>
+      <c r="B61" t="s">
+        <v>26</v>
+      </c>
+      <c r="C61" t="s">
+        <v>198</v>
+      </c>
+      <c r="D61" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A62" s="5">
+        <v>61</v>
+      </c>
+      <c r="B62" t="s">
+        <v>27</v>
+      </c>
+      <c r="C62" t="s">
+        <v>51</v>
+      </c>
+      <c r="D62" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A63" s="5">
+        <v>62</v>
+      </c>
+      <c r="B63" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A64" s="5">
+        <v>63</v>
+      </c>
+      <c r="B64" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A65" s="5">
+        <v>64</v>
+      </c>
+      <c r="B65" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6222BCFE-8BCF-40E1-9440-9F508A532375}">
   <dimension ref="A1:G49"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1677,7 +2357,7 @@
     <col min="4" max="4" width="16.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>89</v>
       </c>
@@ -1690,8 +2370,11 @@
       <c r="D1" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E1" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1699,7 +2382,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1707,7 +2390,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1721,7 +2404,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1735,7 +2418,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1749,7 +2432,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1763,7 +2446,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1777,7 +2460,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1791,7 +2474,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1805,7 +2488,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1819,7 +2502,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1833,7 +2516,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1847,7 +2530,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1861,7 +2544,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1875,7 +2558,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>15</v>
       </c>
@@ -2362,7 +3045,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81371700-F189-4D20-B718-BFF269E87986}">
   <dimension ref="A1:C29"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -2612,7 +3295,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C37"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>

</xml_diff>

<commit_message>
Got 64 pin MSP symbol and footprint and started implementation
</commit_message>
<xml_diff>
--- a/hardware/SwanGanzInterface_V1.1/SwanGanzInterface_v1.1_PinAllocation.xlsx
+++ b/hardware/SwanGanzInterface_V1.1/SwanGanzInterface_v1.1_PinAllocation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ashto\Dev\SeniorDesign_SwanGanz\hardware\SwanGanzInterface_V1.1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3F70114-8A99-475F-A5AB-4C7D0031B5BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75952CA6-9FC2-4DEB-BFA3-A39C1982CA2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="12980" windowHeight="15370" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12710" yWindow="0" windowWidth="12980" windowHeight="15370" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Device Comparision" sheetId="2" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="246">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="271">
   <si>
     <t>Pin</t>
   </si>
@@ -730,9 +730,6 @@
     <t>PENIRQ</t>
   </si>
   <si>
-    <t>PB18 / 1.5</t>
-  </si>
-  <si>
     <t>PB21</t>
   </si>
   <si>
@@ -779,6 +776,84 @@
   </si>
   <si>
     <t>Translated</t>
+  </si>
+  <si>
+    <t>SPEAKER_DAC</t>
+  </si>
+  <si>
+    <t>DAC_OUT</t>
+  </si>
+  <si>
+    <t>UART0_TX</t>
+  </si>
+  <si>
+    <t>UART0_RX</t>
+  </si>
+  <si>
+    <t>FT232_RX</t>
+  </si>
+  <si>
+    <t>FT232_TX</t>
+  </si>
+  <si>
+    <t>FT232_CTS</t>
+  </si>
+  <si>
+    <t>FT232_RTS</t>
+  </si>
+  <si>
+    <t>UART0_CTS</t>
+  </si>
+  <si>
+    <t>UART0_RTS</t>
+  </si>
+  <si>
+    <t>A1.1</t>
+  </si>
+  <si>
+    <t>A1.2</t>
+  </si>
+  <si>
+    <t>TOUCH_BUSY</t>
+  </si>
+  <si>
+    <t>SW_UP</t>
+  </si>
+  <si>
+    <t>SW_DOWN</t>
+  </si>
+  <si>
+    <t>DBG 3</t>
+  </si>
+  <si>
+    <t>DBG 4</t>
+  </si>
+  <si>
+    <t>DBG 5</t>
+  </si>
+  <si>
+    <t>DBG 6</t>
+  </si>
+  <si>
+    <t>DBG 2</t>
+  </si>
+  <si>
+    <t>T_LG</t>
+  </si>
+  <si>
+    <t>T_HG</t>
+  </si>
+  <si>
+    <t>Placed</t>
+  </si>
+  <si>
+    <t>LCD_Backlite</t>
+  </si>
+  <si>
+    <t>SPEAKER_CD</t>
+  </si>
+  <si>
+    <t>FT232_RST</t>
   </si>
 </sst>
 </file>
@@ -794,7 +869,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -831,6 +906,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -844,7 +925,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -854,6 +935,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1741,7 +1823,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D113DCF4-3EF2-4E93-9D02-C93F34579EEA}">
-  <dimension ref="A1:D65"/>
+  <dimension ref="A1:E65"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="23.08984375" bestFit="1" customWidth="1"/>
@@ -1749,7 +1831,7 @@
     <col min="4" max="4" width="16.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1762,88 +1844,138 @@
       <c r="D1" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E1" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C2" t="s">
+        <v>268</v>
+      </c>
+      <c r="D2" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="2">
         <v>2</v>
       </c>
       <c r="B3" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C3" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="2">
         <v>3</v>
       </c>
       <c r="B4" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C4" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="2">
         <v>4</v>
       </c>
       <c r="B5" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C5" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="2">
         <v>5</v>
       </c>
       <c r="B6" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C6" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="2">
         <v>6</v>
       </c>
       <c r="B7" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C7" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="2">
         <v>7</v>
       </c>
       <c r="B8" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C8" t="s">
+        <v>269</v>
+      </c>
+      <c r="D8" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="2">
         <v>8</v>
       </c>
       <c r="B9" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C9" t="s">
+        <v>245</v>
+      </c>
+      <c r="D9" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" s="2">
         <v>9</v>
       </c>
       <c r="B10" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C10" t="s">
+        <v>182</v>
+      </c>
+      <c r="D10" t="s">
+        <v>255</v>
+      </c>
+      <c r="E10" s="7"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" s="2">
         <v>10</v>
       </c>
       <c r="B11" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C11" t="s">
+        <v>184</v>
+      </c>
+      <c r="D11" t="s">
+        <v>256</v>
+      </c>
+      <c r="E11" s="7"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -1851,39 +1983,65 @@
         <v>111</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" s="2">
         <v>12</v>
       </c>
       <c r="B13" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C13" t="s">
+        <v>188</v>
+      </c>
+      <c r="D13" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" s="2">
         <v>13</v>
       </c>
       <c r="B14" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C14" t="s">
+        <v>189</v>
+      </c>
+      <c r="D14" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" s="2">
         <v>14</v>
       </c>
       <c r="B15" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C15" t="s">
+        <v>183</v>
+      </c>
+      <c r="D15" t="s">
+        <v>190</v>
+      </c>
+      <c r="E15" s="7"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" s="2">
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+        <v>164</v>
+      </c>
+      <c r="C16" t="s">
+        <v>185</v>
+      </c>
+      <c r="D16" t="s">
+        <v>191</v>
+      </c>
+      <c r="E16" s="7"/>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -1891,55 +2049,91 @@
         <v>165</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="4">
         <v>17</v>
       </c>
       <c r="B18" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C18" t="s">
+        <v>175</v>
+      </c>
+      <c r="D18" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="4">
         <v>18</v>
       </c>
       <c r="B19" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C19" t="s">
+        <v>258</v>
+      </c>
+      <c r="D19" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="4">
         <v>19</v>
       </c>
       <c r="B20" t="s">
         <v>166</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C20" t="s">
+        <v>259</v>
+      </c>
+      <c r="D20" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="4">
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+        <v>229</v>
+      </c>
+      <c r="C21" t="s">
+        <v>53</v>
+      </c>
+      <c r="D21" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="4">
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+        <v>230</v>
+      </c>
+      <c r="C22" t="s">
+        <v>192</v>
+      </c>
+      <c r="D22" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="4">
         <v>22</v>
       </c>
       <c r="B23" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C23" t="s">
+        <v>193</v>
+      </c>
+      <c r="D23" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" s="4">
         <v>23</v>
       </c>
@@ -1947,23 +2141,29 @@
         <v>167</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="4">
         <v>24</v>
       </c>
       <c r="B25" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C25" t="s">
+        <v>174</v>
+      </c>
+      <c r="D25" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" s="4">
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" s="4">
         <v>26</v>
       </c>
@@ -1971,47 +2171,73 @@
         <v>117</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" s="4">
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+        <v>232</v>
+      </c>
+      <c r="C28" t="s">
+        <v>251</v>
+      </c>
+      <c r="D28" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" s="4">
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+        <v>233</v>
+      </c>
+      <c r="C29" t="s">
+        <v>252</v>
+      </c>
+      <c r="D29" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" s="4">
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" s="4">
         <v>30</v>
       </c>
       <c r="B31" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C31" t="s">
+        <v>265</v>
+      </c>
+      <c r="D31" t="s">
+        <v>181</v>
+      </c>
+      <c r="E31" s="7"/>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" s="4">
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+        <v>235</v>
+      </c>
+      <c r="C32" t="s">
+        <v>266</v>
+      </c>
+      <c r="D32" t="s">
+        <v>180</v>
+      </c>
+      <c r="E32" s="7"/>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="4">
         <v>32</v>
       </c>
@@ -2021,8 +2247,12 @@
       <c r="C33" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D33" t="s">
+        <v>94</v>
+      </c>
+      <c r="E33" s="7"/>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="6">
         <v>33</v>
       </c>
@@ -2030,39 +2260,67 @@
         <v>157</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="6">
         <v>34</v>
       </c>
       <c r="B35" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C35" t="s">
+        <v>249</v>
+      </c>
+      <c r="D35" t="s">
+        <v>248</v>
+      </c>
+      <c r="E35" s="7"/>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" s="6">
         <v>35</v>
       </c>
       <c r="B36" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C36" t="s">
+        <v>250</v>
+      </c>
+      <c r="D36" t="s">
+        <v>247</v>
+      </c>
+      <c r="E36" s="7"/>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="6">
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+        <v>236</v>
+      </c>
+      <c r="C37" t="s">
+        <v>270</v>
+      </c>
+      <c r="D37" t="s">
+        <v>179</v>
+      </c>
+      <c r="E37" s="7"/>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="6">
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+        <v>237</v>
+      </c>
+      <c r="C38" t="s">
+        <v>151</v>
+      </c>
+      <c r="D38" t="s">
+        <v>178</v>
+      </c>
+      <c r="E38" s="7"/>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" s="6">
         <v>38</v>
       </c>
@@ -2072,8 +2330,12 @@
       <c r="C39" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D39" t="s">
+        <v>97</v>
+      </c>
+      <c r="E39" s="7"/>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="6">
         <v>39</v>
       </c>
@@ -2081,7 +2343,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" s="6">
         <v>40</v>
       </c>
@@ -2091,8 +2353,12 @@
       <c r="C41" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D41" t="s">
+        <v>98</v>
+      </c>
+      <c r="E41" s="7"/>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" s="6">
         <v>41</v>
       </c>
@@ -2102,16 +2368,27 @@
       <c r="C42" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D42" t="s">
+        <v>99</v>
+      </c>
+      <c r="E42" s="7"/>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" s="6">
         <v>42</v>
       </c>
       <c r="B43" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C43" t="s">
+        <v>124</v>
+      </c>
+      <c r="D43" t="s">
+        <v>124</v>
+      </c>
+      <c r="E43" s="7"/>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" s="6">
         <v>43</v>
       </c>
@@ -2119,7 +2396,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" s="6">
         <v>44</v>
       </c>
@@ -2127,7 +2404,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" s="6">
         <v>45</v>
       </c>
@@ -2137,8 +2414,12 @@
       <c r="C46" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D46" t="s">
+        <v>173</v>
+      </c>
+      <c r="E46" s="7"/>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" s="6">
         <v>46</v>
       </c>
@@ -2148,8 +2429,12 @@
       <c r="C47" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D47" t="s">
+        <v>122</v>
+      </c>
+      <c r="E47" s="7"/>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" s="6">
         <v>47</v>
       </c>
@@ -2196,13 +2481,25 @@
       <c r="B53" t="s">
         <v>23</v>
       </c>
+      <c r="C53" t="s">
+        <v>257</v>
+      </c>
+      <c r="D53" t="s">
+        <v>178</v>
+      </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A54" s="5">
         <v>53</v>
       </c>
       <c r="B54" t="s">
-        <v>239</v>
+        <v>238</v>
+      </c>
+      <c r="C54" t="s">
+        <v>228</v>
+      </c>
+      <c r="D54" t="s">
+        <v>178</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.35">
@@ -2216,7 +2513,7 @@
         <v>226</v>
       </c>
       <c r="D55" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.35">
@@ -2286,7 +2583,7 @@
         <v>200</v>
       </c>
       <c r="D60" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.35">
@@ -2314,7 +2611,7 @@
         <v>51</v>
       </c>
       <c r="D62" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.35">
@@ -2322,7 +2619,13 @@
         <v>62</v>
       </c>
       <c r="B63" t="s">
-        <v>240</v>
+        <v>239</v>
+      </c>
+      <c r="C63" t="s">
+        <v>47</v>
+      </c>
+      <c r="D63" t="s">
+        <v>178</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.35">
@@ -2330,15 +2633,27 @@
         <v>63</v>
       </c>
       <c r="B64" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
+        <v>240</v>
+      </c>
+      <c r="C64" t="s">
+        <v>55</v>
+      </c>
+      <c r="D64" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A65" s="5">
         <v>64</v>
       </c>
       <c r="B65" t="s">
         <v>28</v>
+      </c>
+      <c r="C65" t="s">
+        <v>54</v>
+      </c>
+      <c r="D65" t="s">
+        <v>179</v>
       </c>
     </row>
   </sheetData>
@@ -2371,7 +2686,7 @@
         <v>156</v>
       </c>
       <c r="E1" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
@@ -2417,6 +2732,7 @@
       <c r="D5" t="s">
         <v>97</v>
       </c>
+      <c r="E5" s="7"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6">
@@ -2445,6 +2761,7 @@
       <c r="D7" t="s">
         <v>98</v>
       </c>
+      <c r="E7" s="7"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8">
@@ -2459,6 +2776,7 @@
       <c r="D8" t="s">
         <v>99</v>
       </c>
+      <c r="E8" s="7"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9">
@@ -2473,6 +2791,7 @@
       <c r="D9" t="s">
         <v>124</v>
       </c>
+      <c r="E9" s="7"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10">
@@ -2515,6 +2834,7 @@
       <c r="D12" t="s">
         <v>173</v>
       </c>
+      <c r="E12" s="7"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13">
@@ -2529,6 +2849,7 @@
       <c r="D13" t="s">
         <v>122</v>
       </c>
+      <c r="E13" s="7"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14">
@@ -2557,6 +2878,7 @@
       <c r="D15" t="s">
         <v>214</v>
       </c>
+      <c r="E15" s="7"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16">
@@ -2571,6 +2893,7 @@
       <c r="D16" t="s">
         <v>215</v>
       </c>
+      <c r="E16" s="7"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17">
@@ -2585,6 +2908,7 @@
       <c r="D17" t="s">
         <v>202</v>
       </c>
+      <c r="E17" s="7"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18">
@@ -2599,6 +2923,7 @@
       <c r="D18" t="s">
         <v>203</v>
       </c>
+      <c r="E18" s="7"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19">
@@ -2627,6 +2952,7 @@
       <c r="D20" t="s">
         <v>209</v>
       </c>
+      <c r="E20" s="7"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21">
@@ -2641,6 +2967,7 @@
       <c r="D21" t="s">
         <v>201</v>
       </c>
+      <c r="E21" s="7"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22">
@@ -2655,6 +2982,7 @@
       <c r="D22" t="s">
         <v>199</v>
       </c>
+      <c r="E22" s="7"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23">
@@ -2669,6 +2997,7 @@
       <c r="D23" t="s">
         <v>197</v>
       </c>
+      <c r="E23" s="7"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24">
@@ -2683,6 +3012,7 @@
       <c r="D24" t="s">
         <v>196</v>
       </c>
+      <c r="E24" s="7"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25">
@@ -2697,6 +3027,7 @@
       <c r="D25" t="s">
         <v>178</v>
       </c>
+      <c r="E25" s="7"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26">
@@ -2711,6 +3042,7 @@
       <c r="D26" t="s">
         <v>179</v>
       </c>
+      <c r="E26" s="7"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27">
@@ -2725,6 +3057,7 @@
       <c r="D27" t="s">
         <v>178</v>
       </c>
+      <c r="E27" s="7"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28">
@@ -2739,6 +3072,7 @@
       <c r="D28" t="s">
         <v>222</v>
       </c>
+      <c r="E28" s="7"/>
       <c r="F28" t="s">
         <v>205</v>
       </c>
@@ -2759,6 +3093,7 @@
       <c r="D29" t="s">
         <v>223</v>
       </c>
+      <c r="E29" s="7"/>
       <c r="F29" t="s">
         <v>206</v>
       </c>
@@ -2779,6 +3114,7 @@
       <c r="D30" t="s">
         <v>225</v>
       </c>
+      <c r="E30" s="7"/>
       <c r="F30" t="s">
         <v>207</v>
       </c>
@@ -2799,6 +3135,7 @@
       <c r="D31" t="s">
         <v>210</v>
       </c>
+      <c r="E31" s="7"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32">
@@ -2813,8 +3150,9 @@
       <c r="D32" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E32" s="7"/>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>32</v>
       </c>
@@ -2822,7 +3160,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>33</v>
       </c>
@@ -2835,8 +3173,9 @@
       <c r="D34" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E34" s="7"/>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>34</v>
       </c>
@@ -2849,8 +3188,9 @@
       <c r="D35" t="s">
         <v>188</v>
       </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E35" s="7"/>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>35</v>
       </c>
@@ -2863,8 +3203,9 @@
       <c r="D36" t="s">
         <v>189</v>
       </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E36" s="7"/>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>36</v>
       </c>
@@ -2877,8 +3218,9 @@
       <c r="D37" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E37" s="7"/>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>37</v>
       </c>
@@ -2891,8 +3233,9 @@
       <c r="D38" t="s">
         <v>191</v>
       </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E38" s="7"/>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>38</v>
       </c>
@@ -2905,8 +3248,9 @@
       <c r="D39" t="s">
         <v>212</v>
       </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E39" s="7"/>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>39</v>
       </c>
@@ -2919,8 +3263,9 @@
       <c r="D40" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E40" s="7"/>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>40</v>
       </c>
@@ -2933,8 +3278,9 @@
       <c r="D41" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E41" s="7"/>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>41</v>
       </c>
@@ -2947,8 +3293,9 @@
       <c r="D42" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E42" s="7"/>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>42</v>
       </c>
@@ -2961,8 +3308,9 @@
       <c r="D43" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E43" s="7"/>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>43</v>
       </c>
@@ -2975,8 +3323,9 @@
       <c r="D44" t="s">
         <v>174</v>
       </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E44" s="7"/>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45">
         <v>44</v>
       </c>
@@ -2989,8 +3338,9 @@
       <c r="D45" t="s">
         <v>227</v>
       </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E45" s="7"/>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>45</v>
       </c>
@@ -2998,7 +3348,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>46</v>
       </c>
@@ -3011,8 +3361,9 @@
       <c r="D47" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E47" s="7"/>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>47</v>
       </c>
@@ -3025,8 +3376,9 @@
       <c r="D48" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E48" s="7"/>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49">
         <v>48</v>
       </c>
@@ -3039,6 +3391,7 @@
       <c r="D49" t="s">
         <v>94</v>
       </c>
+      <c r="E49" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Added debug pins to touch ic and ft232
</commit_message>
<xml_diff>
--- a/hardware/SwanGanzInterface_V1.1/SwanGanzInterface_v1.1_PinAllocation.xlsx
+++ b/hardware/SwanGanzInterface_V1.1/SwanGanzInterface_v1.1_PinAllocation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ashto\Dev\SeniorDesign_SwanGanz\hardware\SwanGanzInterface_V1.1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75952CA6-9FC2-4DEB-BFA3-A39C1982CA2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8B6E8C7-3482-47CF-B3E9-48886D89D80F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12710" yWindow="0" windowWidth="12980" windowHeight="15370" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Device Comparision" sheetId="2" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="271">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="273">
   <si>
     <t>Pin</t>
   </si>
@@ -736,9 +736,6 @@
     <t>PB22</t>
   </si>
   <si>
-    <t>PA23 / A0.3</t>
-  </si>
-  <si>
     <t>PB25 / A0.4</t>
   </si>
   <si>
@@ -823,21 +820,6 @@
     <t>SW_DOWN</t>
   </si>
   <si>
-    <t>DBG 3</t>
-  </si>
-  <si>
-    <t>DBG 4</t>
-  </si>
-  <si>
-    <t>DBG 5</t>
-  </si>
-  <si>
-    <t>DBG 6</t>
-  </si>
-  <si>
-    <t>DBG 2</t>
-  </si>
-  <si>
     <t>T_LG</t>
   </si>
   <si>
@@ -854,6 +836,30 @@
   </si>
   <si>
     <t>FT232_RST</t>
+  </si>
+  <si>
+    <t>DBG1</t>
+  </si>
+  <si>
+    <t>DBG2</t>
+  </si>
+  <si>
+    <t>DBG3</t>
+  </si>
+  <si>
+    <t>DBG4</t>
+  </si>
+  <si>
+    <t>DBG5</t>
+  </si>
+  <si>
+    <t>DBG6</t>
+  </si>
+  <si>
+    <t>DBG7</t>
+  </si>
+  <si>
+    <t>DBG8</t>
   </si>
 </sst>
 </file>
@@ -1845,7 +1851,7 @@
         <v>156</v>
       </c>
       <c r="E1" t="s">
-        <v>267</v>
+        <v>261</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
@@ -1856,7 +1862,7 @@
         <v>29</v>
       </c>
       <c r="C2" t="s">
-        <v>268</v>
+        <v>262</v>
       </c>
       <c r="D2" t="s">
         <v>179</v>
@@ -1870,7 +1876,7 @@
         <v>161</v>
       </c>
       <c r="C3" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
@@ -1881,7 +1887,7 @@
         <v>30</v>
       </c>
       <c r="C4" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
@@ -1892,7 +1898,7 @@
         <v>31</v>
       </c>
       <c r="C5" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
@@ -1903,7 +1909,7 @@
         <v>162</v>
       </c>
       <c r="C6" t="s">
-        <v>262</v>
+        <v>268</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
@@ -1914,7 +1920,7 @@
         <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
@@ -1925,7 +1931,7 @@
         <v>107</v>
       </c>
       <c r="C8" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
       <c r="D8" t="s">
         <v>179</v>
@@ -1939,10 +1945,10 @@
         <v>108</v>
       </c>
       <c r="C9" t="s">
+        <v>244</v>
+      </c>
+      <c r="D9" t="s">
         <v>245</v>
-      </c>
-      <c r="D9" t="s">
-        <v>246</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
@@ -1956,7 +1962,7 @@
         <v>182</v>
       </c>
       <c r="D10" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="E10" s="7"/>
     </row>
@@ -1971,7 +1977,7 @@
         <v>184</v>
       </c>
       <c r="D11" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E11" s="7"/>
     </row>
@@ -2071,10 +2077,7 @@
         <v>115</v>
       </c>
       <c r="C19" t="s">
-        <v>258</v>
-      </c>
-      <c r="D19" t="s">
-        <v>178</v>
+        <v>270</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
@@ -2085,7 +2088,7 @@
         <v>166</v>
       </c>
       <c r="C20" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="D20" t="s">
         <v>178</v>
@@ -2099,7 +2102,7 @@
         <v>229</v>
       </c>
       <c r="C21" t="s">
-        <v>53</v>
+        <v>258</v>
       </c>
       <c r="D21" t="s">
         <v>178</v>
@@ -2113,10 +2116,10 @@
         <v>230</v>
       </c>
       <c r="C22" t="s">
-        <v>192</v>
+        <v>53</v>
       </c>
       <c r="D22" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
@@ -2127,7 +2130,7 @@
         <v>37</v>
       </c>
       <c r="C23" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D23" t="s">
         <v>179</v>
@@ -2140,6 +2143,12 @@
       <c r="B24" t="s">
         <v>167</v>
       </c>
+      <c r="C24" t="s">
+        <v>193</v>
+      </c>
+      <c r="D24" t="s">
+        <v>179</v>
+      </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="4">
@@ -2160,7 +2169,10 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>231</v>
+        <v>118</v>
+      </c>
+      <c r="C26" t="s">
+        <v>271</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.35">
@@ -2170,19 +2182,22 @@
       <c r="B27" t="s">
         <v>117</v>
       </c>
+      <c r="C27" t="s">
+        <v>272</v>
+      </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" s="4">
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C28" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="D28" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.35">
@@ -2190,13 +2205,13 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C29" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D29" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
@@ -2204,7 +2219,7 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.35">
@@ -2215,7 +2230,7 @@
         <v>92</v>
       </c>
       <c r="C31" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
       <c r="D31" t="s">
         <v>181</v>
@@ -2227,10 +2242,10 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C32" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="D32" t="s">
         <v>180</v>
@@ -2268,10 +2283,10 @@
         <v>96</v>
       </c>
       <c r="C35" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D35" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E35" s="7"/>
     </row>
@@ -2283,10 +2298,10 @@
         <v>16</v>
       </c>
       <c r="C36" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D36" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E36" s="7"/>
     </row>
@@ -2295,10 +2310,10 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C37" t="s">
-        <v>270</v>
+        <v>264</v>
       </c>
       <c r="D37" t="s">
         <v>179</v>
@@ -2310,7 +2325,7 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C38" t="s">
         <v>151</v>
@@ -2482,7 +2497,7 @@
         <v>23</v>
       </c>
       <c r="C53" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="D53" t="s">
         <v>178</v>
@@ -2493,7 +2508,7 @@
         <v>53</v>
       </c>
       <c r="B54" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C54" t="s">
         <v>228</v>
@@ -2513,7 +2528,7 @@
         <v>226</v>
       </c>
       <c r="D55" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.35">
@@ -2583,7 +2598,7 @@
         <v>200</v>
       </c>
       <c r="D60" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.35">
@@ -2611,7 +2626,7 @@
         <v>51</v>
       </c>
       <c r="D62" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.35">
@@ -2619,7 +2634,7 @@
         <v>62</v>
       </c>
       <c r="B63" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C63" t="s">
         <v>47</v>
@@ -2633,7 +2648,7 @@
         <v>63</v>
       </c>
       <c r="B64" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C64" t="s">
         <v>55</v>
@@ -2686,7 +2701,7 @@
         <v>156</v>
       </c>
       <c r="E1" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Button pin allocation, layout of power and ft, general layout
</commit_message>
<xml_diff>
--- a/hardware/SwanGanzInterface_V1.1/SwanGanzInterface_v1.1_PinAllocation.xlsx
+++ b/hardware/SwanGanzInterface_V1.1/SwanGanzInterface_v1.1_PinAllocation.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ashto\Dev\SeniorDesign_SwanGanz\hardware\SwanGanzInterface_V1.1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ashton\Dev\SeniorDesign_SwanGanz\hardware\SwanGanzInterface_V1.1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C3796D3-C01D-42FA-8D26-40930A2C2E89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9457FF07-95E9-4349-B5A6-92EB31670F23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Device Comparision" sheetId="2" r:id="rId1"/>
@@ -1223,17 +1223,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7AC523F-0BD7-4B46-B60C-E63BF843905A}">
   <dimension ref="A1:L7"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.26953125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.90625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.54296875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.453125" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="13.7265625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>60</v>
       </c>
@@ -1271,7 +1271,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>59</v>
       </c>
@@ -1309,7 +1309,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>61</v>
       </c>
@@ -1347,7 +1347,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>62</v>
       </c>
@@ -1385,7 +1385,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>63</v>
       </c>
@@ -1423,7 +1423,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>64</v>
       </c>
@@ -1461,7 +1461,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>65</v>
       </c>
@@ -1507,17 +1507,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74AC5E4A-A5B7-4659-9F92-160B4C389A21}">
   <dimension ref="A1:F24"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.6328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.6328125" customWidth="1"/>
-    <col min="3" max="3" width="47.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="40.6328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.54296875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" customWidth="1"/>
+    <col min="3" max="3" width="47.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="40.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>119</v>
       </c>
@@ -1537,7 +1537,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>169</v>
       </c>
@@ -1555,7 +1555,7 @@
       </c>
       <c r="F2" s="3"/>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>122</v>
       </c>
@@ -1573,7 +1573,7 @@
       </c>
       <c r="F3" s="3"/>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>124</v>
       </c>
@@ -1585,7 +1585,7 @@
       </c>
       <c r="F4" s="3"/>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>128</v>
       </c>
@@ -1597,7 +1597,7 @@
       </c>
       <c r="F5" s="3"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>129</v>
       </c>
@@ -1609,7 +1609,7 @@
       </c>
       <c r="F6" s="3"/>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>130</v>
       </c>
@@ -1621,7 +1621,7 @@
       </c>
       <c r="F7" s="3"/>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>51</v>
       </c>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="F8" s="3"/>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>49</v>
       </c>
@@ -1645,7 +1645,7 @@
       </c>
       <c r="F9" s="3"/>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>136</v>
       </c>
@@ -1657,7 +1657,7 @@
       </c>
       <c r="F10" s="3"/>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>48</v>
       </c>
@@ -1669,7 +1669,7 @@
       </c>
       <c r="F11" s="3"/>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>54</v>
       </c>
@@ -1681,7 +1681,7 @@
       </c>
       <c r="F12" s="3"/>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>55</v>
       </c>
@@ -1693,7 +1693,7 @@
       </c>
       <c r="F13" s="3"/>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>47</v>
       </c>
@@ -1705,7 +1705,7 @@
       </c>
       <c r="F14" s="3"/>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>140</v>
       </c>
@@ -1717,7 +1717,7 @@
       </c>
       <c r="F15" s="3"/>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>144</v>
       </c>
@@ -1729,7 +1729,7 @@
       </c>
       <c r="F16" s="3"/>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>146</v>
       </c>
@@ -1741,7 +1741,7 @@
       </c>
       <c r="F17" s="3"/>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>151</v>
       </c>
@@ -1753,7 +1753,7 @@
       </c>
       <c r="F18" s="3"/>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>148</v>
       </c>
@@ -1765,7 +1765,7 @@
       </c>
       <c r="F19" s="3"/>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>40</v>
       </c>
@@ -1777,7 +1777,7 @@
       </c>
       <c r="F20" s="3"/>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>127</v>
       </c>
@@ -1789,7 +1789,7 @@
       </c>
       <c r="F21" s="3"/>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>189</v>
       </c>
@@ -1801,7 +1801,7 @@
       </c>
       <c r="F22" s="3"/>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>188</v>
       </c>
@@ -1813,7 +1813,7 @@
       </c>
       <c r="F23" s="3"/>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>154</v>
       </c>
@@ -1830,14 +1830,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D113DCF4-3EF2-4E93-9D02-C93F34579EEA}">
   <dimension ref="A1:E65"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="23.08984375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1854,7 +1854,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -1869,7 +1869,7 @@
       </c>
       <c r="E2" s="2"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -1884,7 +1884,7 @@
       </c>
       <c r="E3" s="2"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -1899,7 +1899,7 @@
       </c>
       <c r="E4" s="2"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -1914,7 +1914,7 @@
       </c>
       <c r="E5" s="2"/>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -1929,7 +1929,7 @@
       </c>
       <c r="E6" s="2"/>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -1944,7 +1944,7 @@
       </c>
       <c r="E7" s="2"/>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -1959,7 +1959,7 @@
       </c>
       <c r="E8" s="2"/>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -1974,7 +1974,7 @@
       </c>
       <c r="E9" s="2"/>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -1989,7 +1989,7 @@
       </c>
       <c r="E10" s="2"/>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -2004,16 +2004,22 @@
       </c>
       <c r="E11" s="2"/>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>11</v>
       </c>
       <c r="B12" t="s">
         <v>111</v>
       </c>
+      <c r="C12" t="s">
+        <v>192</v>
+      </c>
+      <c r="D12" t="s">
+        <v>179</v>
+      </c>
       <c r="E12" s="2"/>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -2028,7 +2034,7 @@
       </c>
       <c r="E13" s="2"/>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -2043,7 +2049,7 @@
       </c>
       <c r="E14" s="2"/>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -2058,7 +2064,7 @@
       </c>
       <c r="E15" s="2"/>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -2073,16 +2079,22 @@
       </c>
       <c r="E16" s="2"/>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>16</v>
       </c>
       <c r="B17" t="s">
         <v>165</v>
       </c>
+      <c r="C17" t="s">
+        <v>193</v>
+      </c>
+      <c r="D17" t="s">
+        <v>179</v>
+      </c>
       <c r="E17" s="2"/>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="4">
         <v>17</v>
       </c>
@@ -2097,7 +2109,7 @@
       </c>
       <c r="E18" s="2"/>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="4">
         <v>18</v>
       </c>
@@ -2109,7 +2121,7 @@
       </c>
       <c r="E19" s="2"/>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="4">
         <v>19</v>
       </c>
@@ -2124,7 +2136,7 @@
       </c>
       <c r="E20" s="2"/>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="4">
         <v>20</v>
       </c>
@@ -2139,7 +2151,7 @@
       </c>
       <c r="E21" s="2"/>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="4">
         <v>21</v>
       </c>
@@ -2154,37 +2166,25 @@
       </c>
       <c r="E22" s="2"/>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="4">
         <v>22</v>
       </c>
       <c r="B23" t="s">
         <v>37</v>
       </c>
-      <c r="C23" t="s">
-        <v>192</v>
-      </c>
-      <c r="D23" t="s">
-        <v>179</v>
-      </c>
       <c r="E23" s="2"/>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="4">
         <v>23</v>
       </c>
       <c r="B24" t="s">
         <v>167</v>
       </c>
-      <c r="C24" t="s">
-        <v>193</v>
-      </c>
-      <c r="D24" t="s">
-        <v>179</v>
-      </c>
       <c r="E24" s="2"/>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="4">
         <v>24</v>
       </c>
@@ -2199,7 +2199,7 @@
       </c>
       <c r="E25" s="2"/>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="4">
         <v>25</v>
       </c>
@@ -2211,7 +2211,7 @@
       </c>
       <c r="E26" s="2"/>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="4">
         <v>26</v>
       </c>
@@ -2223,7 +2223,7 @@
       </c>
       <c r="E27" s="2"/>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="4">
         <v>27</v>
       </c>
@@ -2238,7 +2238,7 @@
       </c>
       <c r="E28" s="2"/>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="4">
         <v>28</v>
       </c>
@@ -2253,7 +2253,7 @@
       </c>
       <c r="E29" s="2"/>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="4">
         <v>29</v>
       </c>
@@ -2262,7 +2262,7 @@
       </c>
       <c r="E30" s="2"/>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="4">
         <v>30</v>
       </c>
@@ -2277,7 +2277,7 @@
       </c>
       <c r="E31" s="2"/>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="4">
         <v>31</v>
       </c>
@@ -2292,7 +2292,7 @@
       </c>
       <c r="E32" s="2"/>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="4">
         <v>32</v>
       </c>
@@ -2307,7 +2307,7 @@
       </c>
       <c r="E33" s="2"/>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="6">
         <v>33</v>
       </c>
@@ -2316,7 +2316,7 @@
       </c>
       <c r="E34" s="2"/>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="6">
         <v>34</v>
       </c>
@@ -2331,7 +2331,7 @@
       </c>
       <c r="E35" s="2"/>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="6">
         <v>35</v>
       </c>
@@ -2346,7 +2346,7 @@
       </c>
       <c r="E36" s="2"/>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="6">
         <v>36</v>
       </c>
@@ -2361,7 +2361,7 @@
       </c>
       <c r="E37" s="2"/>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="6">
         <v>37</v>
       </c>
@@ -2376,7 +2376,7 @@
       </c>
       <c r="E38" s="2"/>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="6">
         <v>38</v>
       </c>
@@ -2391,7 +2391,7 @@
       </c>
       <c r="E39" s="2"/>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="6">
         <v>39</v>
       </c>
@@ -2400,7 +2400,7 @@
       </c>
       <c r="E40" s="2"/>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="6">
         <v>40</v>
       </c>
@@ -2415,7 +2415,7 @@
       </c>
       <c r="E41" s="2"/>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="6">
         <v>41</v>
       </c>
@@ -2430,7 +2430,7 @@
       </c>
       <c r="E42" s="2"/>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="6">
         <v>42</v>
       </c>
@@ -2445,7 +2445,7 @@
       </c>
       <c r="E43" s="2"/>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="6">
         <v>43</v>
       </c>
@@ -2454,7 +2454,7 @@
       </c>
       <c r="E44" s="2"/>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="6">
         <v>44</v>
       </c>
@@ -2463,7 +2463,7 @@
       </c>
       <c r="E45" s="2"/>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="6">
         <v>45</v>
       </c>
@@ -2478,7 +2478,7 @@
       </c>
       <c r="E46" s="2"/>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="6">
         <v>46</v>
       </c>
@@ -2493,7 +2493,7 @@
       </c>
       <c r="E47" s="2"/>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="6">
         <v>47</v>
       </c>
@@ -2502,7 +2502,7 @@
       </c>
       <c r="E48" s="2"/>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="6">
         <v>48</v>
       </c>
@@ -2511,7 +2511,7 @@
       </c>
       <c r="E49" s="2"/>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="5">
         <v>49</v>
       </c>
@@ -2520,7 +2520,7 @@
       </c>
       <c r="E50" s="2"/>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="5">
         <v>50</v>
       </c>
@@ -2529,7 +2529,7 @@
       </c>
       <c r="E51" s="2"/>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="5">
         <v>51</v>
       </c>
@@ -2538,7 +2538,7 @@
       </c>
       <c r="E52" s="2"/>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="5">
         <v>52</v>
       </c>
@@ -2553,7 +2553,7 @@
       </c>
       <c r="E53" s="2"/>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="5">
         <v>53</v>
       </c>
@@ -2568,7 +2568,7 @@
       </c>
       <c r="E54" s="2"/>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="5">
         <v>54</v>
       </c>
@@ -2583,7 +2583,7 @@
       </c>
       <c r="E55" s="2"/>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="5">
         <v>55</v>
       </c>
@@ -2598,7 +2598,7 @@
       </c>
       <c r="E56" s="2"/>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="5">
         <v>56</v>
       </c>
@@ -2613,7 +2613,7 @@
       </c>
       <c r="E57" s="2"/>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="5">
         <v>57</v>
       </c>
@@ -2628,7 +2628,7 @@
       </c>
       <c r="E58" s="2"/>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="5">
         <v>58</v>
       </c>
@@ -2643,7 +2643,7 @@
       </c>
       <c r="E59" s="2"/>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="5">
         <v>59</v>
       </c>
@@ -2658,7 +2658,7 @@
       </c>
       <c r="E60" s="2"/>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="5">
         <v>60</v>
       </c>
@@ -2673,7 +2673,7 @@
       </c>
       <c r="E61" s="2"/>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="5">
         <v>61</v>
       </c>
@@ -2688,7 +2688,7 @@
       </c>
       <c r="E62" s="2"/>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="5">
         <v>62</v>
       </c>
@@ -2703,7 +2703,7 @@
       </c>
       <c r="E63" s="2"/>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="5">
         <v>63</v>
       </c>
@@ -2718,7 +2718,7 @@
       </c>
       <c r="E64" s="2"/>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="5">
         <v>64</v>
       </c>
@@ -2741,15 +2741,15 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6222BCFE-8BCF-40E1-9440-9F508A532375}">
   <dimension ref="A1:G49"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.6328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.08984375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.36328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>89</v>
       </c>
@@ -2766,7 +2766,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2774,7 +2774,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -2782,7 +2782,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -2796,7 +2796,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -2811,7 +2811,7 @@
       </c>
       <c r="E5" s="7"/>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -2825,7 +2825,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -2840,7 +2840,7 @@
       </c>
       <c r="E7" s="7"/>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -2855,7 +2855,7 @@
       </c>
       <c r="E8" s="7"/>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -2870,7 +2870,7 @@
       </c>
       <c r="E9" s="7"/>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -2884,7 +2884,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -2898,7 +2898,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -2913,7 +2913,7 @@
       </c>
       <c r="E12" s="7"/>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -2928,7 +2928,7 @@
       </c>
       <c r="E13" s="7"/>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -2942,7 +2942,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -2957,7 +2957,7 @@
       </c>
       <c r="E15" s="7"/>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -2972,7 +2972,7 @@
       </c>
       <c r="E16" s="7"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -2987,7 +2987,7 @@
       </c>
       <c r="E17" s="7"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
@@ -3002,7 +3002,7 @@
       </c>
       <c r="E18" s="7"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -3016,7 +3016,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
@@ -3031,7 +3031,7 @@
       </c>
       <c r="E20" s="7"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -3046,7 +3046,7 @@
       </c>
       <c r="E21" s="7"/>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
@@ -3061,7 +3061,7 @@
       </c>
       <c r="E22" s="7"/>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
@@ -3076,7 +3076,7 @@
       </c>
       <c r="E23" s="7"/>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
@@ -3091,7 +3091,7 @@
       </c>
       <c r="E24" s="7"/>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
@@ -3106,7 +3106,7 @@
       </c>
       <c r="E25" s="7"/>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
@@ -3121,7 +3121,7 @@
       </c>
       <c r="E26" s="7"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
@@ -3136,7 +3136,7 @@
       </c>
       <c r="E27" s="7"/>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
@@ -3157,7 +3157,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
@@ -3178,7 +3178,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>29</v>
       </c>
@@ -3199,7 +3199,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>30</v>
       </c>
@@ -3214,7 +3214,7 @@
       </c>
       <c r="E31" s="7"/>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>31</v>
       </c>
@@ -3229,7 +3229,7 @@
       </c>
       <c r="E32" s="7"/>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>32</v>
       </c>
@@ -3237,7 +3237,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>33</v>
       </c>
@@ -3252,7 +3252,7 @@
       </c>
       <c r="E34" s="7"/>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>34</v>
       </c>
@@ -3267,7 +3267,7 @@
       </c>
       <c r="E35" s="7"/>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>35</v>
       </c>
@@ -3282,7 +3282,7 @@
       </c>
       <c r="E36" s="7"/>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>36</v>
       </c>
@@ -3297,7 +3297,7 @@
       </c>
       <c r="E37" s="7"/>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>37</v>
       </c>
@@ -3312,7 +3312,7 @@
       </c>
       <c r="E38" s="7"/>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>38</v>
       </c>
@@ -3327,7 +3327,7 @@
       </c>
       <c r="E39" s="7"/>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>39</v>
       </c>
@@ -3342,7 +3342,7 @@
       </c>
       <c r="E40" s="7"/>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>40</v>
       </c>
@@ -3357,7 +3357,7 @@
       </c>
       <c r="E41" s="7"/>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>41</v>
       </c>
@@ -3372,7 +3372,7 @@
       </c>
       <c r="E42" s="7"/>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>42</v>
       </c>
@@ -3387,7 +3387,7 @@
       </c>
       <c r="E43" s="7"/>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>43</v>
       </c>
@@ -3402,7 +3402,7 @@
       </c>
       <c r="E44" s="7"/>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>44</v>
       </c>
@@ -3417,7 +3417,7 @@
       </c>
       <c r="E45" s="7"/>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>45</v>
       </c>
@@ -3425,7 +3425,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>46</v>
       </c>
@@ -3440,7 +3440,7 @@
       </c>
       <c r="E47" s="7"/>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>47</v>
       </c>
@@ -3455,7 +3455,7 @@
       </c>
       <c r="E48" s="7"/>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>48</v>
       </c>
@@ -3478,14 +3478,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81371700-F189-4D20-B718-BFF269E87986}">
   <dimension ref="A1:C29"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.6328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.08984375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>89</v>
       </c>
@@ -3496,7 +3496,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -3504,7 +3504,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -3512,7 +3512,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -3520,7 +3520,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -3528,7 +3528,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -3536,7 +3536,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -3544,7 +3544,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -3552,7 +3552,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -3560,7 +3560,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -3568,7 +3568,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -3576,7 +3576,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -3584,7 +3584,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -3592,7 +3592,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -3600,7 +3600,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -3608,7 +3608,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -3616,7 +3616,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -3624,7 +3624,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
@@ -3632,7 +3632,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -3640,7 +3640,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
@@ -3648,7 +3648,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -3656,7 +3656,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
@@ -3664,7 +3664,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
@@ -3672,7 +3672,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
@@ -3680,7 +3680,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
@@ -3688,7 +3688,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
@@ -3696,7 +3696,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
@@ -3704,7 +3704,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
@@ -3712,7 +3712,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
@@ -3728,13 +3728,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C37"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3745,7 +3745,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -3756,7 +3756,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -3767,7 +3767,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -3778,7 +3778,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -3789,7 +3789,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -3800,7 +3800,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -3811,7 +3811,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -3822,7 +3822,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -3833,7 +3833,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>10</v>
       </c>
@@ -3844,7 +3844,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -3855,7 +3855,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -3866,7 +3866,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>13</v>
       </c>
@@ -3877,7 +3877,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>14</v>
       </c>
@@ -3888,7 +3888,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>15</v>
       </c>
@@ -3899,7 +3899,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>16</v>
       </c>
@@ -3910,7 +3910,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>17</v>
       </c>
@@ -3921,7 +3921,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>18</v>
       </c>
@@ -3932,7 +3932,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>19</v>
       </c>
@@ -3943,7 +3943,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>20</v>
       </c>
@@ -3954,7 +3954,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>22</v>
       </c>
@@ -3965,7 +3965,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>23</v>
       </c>
@@ -3976,7 +3976,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>24</v>
       </c>
@@ -3987,7 +3987,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>25</v>
       </c>
@@ -3998,7 +3998,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>26</v>
       </c>
@@ -4009,7 +4009,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>27</v>
       </c>
@@ -4020,7 +4020,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>28</v>
       </c>
@@ -4031,7 +4031,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>29</v>
       </c>
@@ -4042,7 +4042,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>30</v>
       </c>
@@ -4053,7 +4053,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>31</v>
       </c>
@@ -4064,7 +4064,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>32</v>
       </c>
@@ -4075,7 +4075,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>33</v>
       </c>
@@ -4086,7 +4086,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>34</v>
       </c>
@@ -4097,7 +4097,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>35</v>
       </c>
@@ -4108,7 +4108,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>37</v>
       </c>
@@ -4119,7 +4119,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>36</v>
       </c>
@@ -4130,7 +4130,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B37" t="s">
         <v>58</v>
       </c>

</xml_diff>